<commit_message>
Update SRX4XX datasheet with latest test data
</commit_message>
<xml_diff>
--- a/public/data/SRX4XX_Datasheet.xlsx
+++ b/public/data/SRX4XX_Datasheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpe-my.sharepoint.com/personal/antony-ruban_alexis_hpe_com/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="313" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A36155C-B35E-4860-8555-938A055F3044}"/>
+  <xr:revisionPtr revIDLastSave="381" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3BF448C6-ACA0-41B6-AF91-530DAF76D438}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="38400" windowHeight="19740" firstSheet="2" activeTab="2" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19740" firstSheet="1" activeTab="2" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
   </bookViews>
   <sheets>
     <sheet name="ISSUES-PR's" sheetId="7" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1061" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1083" uniqueCount="415">
   <si>
     <t>number</t>
   </si>
@@ -678,6 +678,9 @@
     <t>3500 CPS / 1950 Mbps</t>
   </si>
   <si>
+    <t>* Need Additional Port Pair</t>
+  </si>
+  <si>
     <t xml:space="preserve">AppSec + AppQOS with ASC enabled </t>
   </si>
   <si>
@@ -723,6 +726,9 @@
     <t>AppSec + UTM SAV</t>
   </si>
   <si>
+    <t>381 CPS / 211 Mbps</t>
+  </si>
+  <si>
     <t>AppSec + SecIntel+ IDP-Rec + UTM EWF</t>
   </si>
   <si>
@@ -744,6 +750,9 @@
     <t>AppSec + SecIntel+ IDP-Rec + UTM EWF + UTM SAV</t>
   </si>
   <si>
+    <t>307 CPS / 165 Mbps</t>
+  </si>
+  <si>
     <t xml:space="preserve">AppSec + SecIntel+ IDP-Rec + SkyATP Block + DNS </t>
   </si>
   <si>
@@ -766,6 +775,9 @@
   </si>
   <si>
     <t>AppSec + SSL(TLS1.3)</t>
+  </si>
+  <si>
+    <t>125 CPS / 66 Mbps</t>
   </si>
   <si>
     <t xml:space="preserve">AppSec + SSL+ IDP-Recommended policy </t>
@@ -820,54 +832,63 @@
     <t>Firewall + AppSec(Unified policy)</t>
   </si>
   <si>
+    <t>6930 TPS / 3995 Mbps</t>
+  </si>
+  <si>
+    <t>*100 Sessions</t>
+  </si>
+  <si>
     <t>AppSec + IDP-Recommended policy template</t>
   </si>
   <si>
     <t>AppSec + IDP-Rec + UTM EWF(100% cache)</t>
   </si>
   <si>
+    <t>650 TPS / 256 Mbps</t>
+  </si>
+  <si>
+    <t>CPS Performance (Payload: 64B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firewall TCP CPS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">IPv6 Firewall TCP CPS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppSec with ASC enabled CPS </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppSec CPS </t>
+  </si>
+  <si>
+    <t>UTM EWF-100% cache</t>
+  </si>
+  <si>
+    <t>UTM- SAV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppSec + TCPProxy </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppSec + SSL(TLS1.2) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AppSec + SSL(TLS1.3) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UDP/IPSec Throughput </t>
+  </si>
+  <si>
+    <t>Firewall UDP throughput- Packet size 64bytes</t>
+  </si>
+  <si>
+    <t>654.7 KPPS / 440 Mbps</t>
+  </si>
+  <si>
     <t>*400 Sessions</t>
   </si>
   <si>
-    <t>CPS Performance (Payload: 64B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Firewall TCP CPS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">IPv6 Firewall TCP CPS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AppSec with ASC enabled CPS </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AppSec CPS </t>
-  </si>
-  <si>
-    <t>UTM EWF-100% cache</t>
-  </si>
-  <si>
-    <t>UTM- SAV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AppSec + TCPProxy </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AppSec + SSL(TLS1.2) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AppSec + SSL(TLS1.3) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UDP/IPSec Throughput </t>
-  </si>
-  <si>
-    <t>Firewall UDP throughput- Packet size 64bytes</t>
-  </si>
-  <si>
-    <t>654.7 KPPS / 440 Mbps</t>
-  </si>
-  <si>
     <t>Firewall UDP throughput- Packet size IMIX(ratio: 64:7, 570:4, 1518:1)</t>
   </si>
   <si>
@@ -880,9 +901,6 @@
     <t>487.6 KPPS / 6000 Mbps</t>
   </si>
   <si>
-    <t xml:space="preserve">We don’t have another pair of ports connected to this 400 device </t>
-  </si>
-  <si>
     <t>Single flow/session Firewall UDP Throughput- IMIX</t>
   </si>
   <si>
@@ -955,6 +973,9 @@
     <t>IPSec(site-2-site) UDP throughput with IKEv2,PSK,AES-GCM256- Packet size 64bytes</t>
   </si>
   <si>
+    <t>PR 1954277 </t>
+  </si>
+  <si>
     <t>IPSec(site-2-site) UDP throughput with IKEv2,PSK,AES-GCM256- Packet size IMIX(ratio 64:7,570:4,1400:1)</t>
   </si>
   <si>
@@ -1078,7 +1099,7 @@
     <t>Max Sky ATP session capacity</t>
   </si>
   <si>
-    <t>PR</t>
+    <t>PR 1957107</t>
   </si>
   <si>
     <t>Max SSL Inspection sessions(TLS1.2)</t>
@@ -1189,6 +1210,9 @@
   </si>
   <si>
     <t>CPS</t>
+  </si>
+  <si>
+    <t>y</t>
   </si>
   <si>
     <t>Sessions</t>
@@ -4498,13 +4522,16 @@
       <c r="D4" s="4">
         <v>70</v>
       </c>
+      <c r="E4" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="5" spans="1:5" ht="15.6" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="C5" s="4">
         <v>92</v>
@@ -4516,10 +4543,10 @@
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C6" s="1">
         <v>95</v>
@@ -4531,10 +4558,10 @@
     </row>
     <row r="7" spans="1:5" ht="14.45" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="C7" s="4">
         <v>95</v>
@@ -4545,10 +4572,10 @@
     </row>
     <row r="8" spans="1:5" ht="14.1" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C8" s="4">
         <v>91</v>
@@ -4559,10 +4586,10 @@
     </row>
     <row r="9" spans="1:5" ht="15.95">
       <c r="A9" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C9" s="4">
         <v>96</v>
@@ -4573,10 +4600,10 @@
     </row>
     <row r="10" spans="1:5" ht="15.95">
       <c r="A10" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C10" s="4">
         <v>93</v>
@@ -4587,10 +4614,10 @@
     </row>
     <row r="11" spans="1:5" ht="15.95">
       <c r="A11" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C11" s="4">
         <v>93</v>
@@ -4601,18 +4628,24 @@
     </row>
     <row r="12" spans="1:5" ht="15.95">
       <c r="A12" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="59"/>
+        <v>218</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="C12" s="1">
+        <v>93</v>
+      </c>
+      <c r="D12" s="59">
+        <v>45</v>
+      </c>
     </row>
     <row r="13" spans="1:5" ht="15.95">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C13" s="1">
         <v>94</v>
@@ -4623,10 +4656,10 @@
     </row>
     <row r="14" spans="1:5" ht="15.95">
       <c r="A14" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C14" s="4">
         <v>95</v>
@@ -4637,10 +4670,10 @@
     </row>
     <row r="15" spans="1:5" ht="15.95">
       <c r="A15" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C15" s="1">
         <v>95</v>
@@ -4651,18 +4684,24 @@
     </row>
     <row r="16" spans="1:5" ht="15.95">
       <c r="A16" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="4"/>
-    </row>
-    <row r="17" spans="1:4" ht="15.95">
+        <v>226</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="C16" s="46">
+        <v>94</v>
+      </c>
+      <c r="D16" s="4">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="15.95">
       <c r="A17" s="43" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C17" s="7">
         <v>96</v>
@@ -4671,9 +4710,9 @@
         <v>76</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="40.5" customHeight="1">
+    <row r="18" spans="1:5" ht="40.5" customHeight="1">
       <c r="A18" s="38" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B18" s="39" t="s">
         <v>196</v>
@@ -4685,12 +4724,12 @@
         <v>198</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15.95">
+    <row r="19" spans="1:5" ht="15.95">
       <c r="A19" s="22" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B19" s="44" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C19" s="27">
         <v>85</v>
@@ -4699,12 +4738,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="15.95">
+    <row r="20" spans="1:5" ht="15.95">
       <c r="A20" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="C20" s="23">
         <v>90</v>
@@ -4713,20 +4752,26 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="15.95">
+    <row r="21" spans="1:5" ht="15.95">
       <c r="A21" s="2" t="s">
-        <v>232</v>
-      </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="57"/>
-    </row>
-    <row r="22" spans="1:4" ht="15.95">
+        <v>235</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="C21" s="10">
+        <v>92</v>
+      </c>
+      <c r="D21" s="57">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.95">
       <c r="A22" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="C22" s="10">
         <v>90</v>
@@ -4735,12 +4780,12 @@
         <v>69</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15.95">
+    <row r="23" spans="1:5" ht="15.95">
       <c r="A23" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C23" s="10">
         <v>90</v>
@@ -4749,12 +4794,12 @@
         <v>69</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="15.95">
+    <row r="24" spans="1:5" ht="15.95">
       <c r="A24" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="C24" s="10">
         <v>95</v>
@@ -4763,12 +4808,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="15.95">
+    <row r="25" spans="1:5" ht="15.95">
       <c r="A25" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="C25" s="10">
         <v>91</v>
@@ -4777,12 +4822,12 @@
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="15.95">
+    <row r="26" spans="1:5" ht="15.95">
       <c r="A26" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>242</v>
+        <v>246</v>
       </c>
       <c r="C26" s="10">
         <v>93</v>
@@ -4791,12 +4836,12 @@
         <v>59</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.95">
+    <row r="27" spans="1:5" ht="15.95">
       <c r="A27" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C27" s="10">
         <v>92</v>
@@ -4805,12 +4850,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="15.95">
+    <row r="28" spans="1:5" ht="15.95">
       <c r="A28" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="C28" s="10">
         <v>93</v>
@@ -4819,12 +4864,12 @@
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="39" customHeight="1">
+    <row r="29" spans="1:5" ht="39" customHeight="1">
       <c r="A29" s="29" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B29" s="39" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>197</v>
@@ -4833,43 +4878,74 @@
         <v>198</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="15.95">
+    <row r="30" spans="1:5" ht="15.95">
       <c r="A30" s="2" t="s">
-        <v>249</v>
-      </c>
-      <c r="B30" s="4"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="57"/>
-    </row>
-    <row r="31" spans="1:4" ht="15.95">
+        <v>253</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C30" s="47">
+        <v>77</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E30" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" ht="15.95">
       <c r="A31" s="2" t="s">
-        <v>250</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="57"/>
-    </row>
-    <row r="32" spans="1:4" ht="15.95">
+        <v>256</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C31" s="47">
+        <v>77</v>
+      </c>
+      <c r="D31" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E31" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="15.95">
       <c r="A32" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="B32" s="6"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="57"/>
+        <v>257</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="C32" s="47">
+        <v>77</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>255</v>
+      </c>
+      <c r="E32" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="33" spans="1:5" ht="17.45" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="B33" s="6"/>
-      <c r="C33" s="47"/>
+        <v>233</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C33" s="47">
+        <v>93</v>
+      </c>
       <c r="D33" s="24" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="41.25" customHeight="1">
       <c r="A34" s="29" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B34" s="39" t="s">
         <v>196</v>
@@ -4883,7 +4959,7 @@
     </row>
     <row r="35" spans="1:5" ht="15.95">
       <c r="A35" s="2" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B35" s="4">
         <v>20000</v>
@@ -4897,7 +4973,7 @@
     </row>
     <row r="36" spans="1:5" ht="15.95">
       <c r="A36" s="2" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B36" s="4">
         <v>19330</v>
@@ -4911,7 +4987,7 @@
     </row>
     <row r="37" spans="1:5" ht="15.6" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B37" s="4">
         <v>10000</v>
@@ -4925,7 +5001,7 @@
     </row>
     <row r="38" spans="1:5" ht="15.95">
       <c r="A38" s="2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B38" s="4">
         <v>2400</v>
@@ -4939,7 +5015,7 @@
     </row>
     <row r="39" spans="1:5" ht="15.95">
       <c r="A39" s="22" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B39" s="15">
         <v>2250</v>
@@ -4953,15 +5029,21 @@
     </row>
     <row r="40" spans="1:5" ht="15.95">
       <c r="A40" s="22" t="s">
-        <v>259</v>
-      </c>
-      <c r="B40" s="45"/>
-      <c r="C40" s="45"/>
-      <c r="D40" s="15"/>
+        <v>265</v>
+      </c>
+      <c r="B40" s="45">
+        <v>975</v>
+      </c>
+      <c r="C40" s="45">
+        <v>86</v>
+      </c>
+      <c r="D40" s="15">
+        <v>48</v>
+      </c>
     </row>
     <row r="41" spans="1:5" ht="15.95">
       <c r="A41" s="2" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B41" s="4">
         <v>1550</v>
@@ -4975,7 +5057,7 @@
     </row>
     <row r="42" spans="1:5" ht="15.95">
       <c r="A42" s="2" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B42" s="4">
         <v>400</v>
@@ -4989,15 +5071,21 @@
     </row>
     <row r="43" spans="1:5" ht="15.95">
       <c r="A43" s="2" t="s">
-        <v>262</v>
-      </c>
-      <c r="B43" s="4"/>
-      <c r="C43" s="4"/>
-      <c r="D43" s="4"/>
+        <v>268</v>
+      </c>
+      <c r="B43" s="4">
+        <v>175</v>
+      </c>
+      <c r="C43" s="4">
+        <v>87</v>
+      </c>
+      <c r="D43" s="4">
+        <v>70</v>
+      </c>
     </row>
     <row r="44" spans="1:5" ht="32.25" customHeight="1">
       <c r="A44" s="29" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B44" s="39" t="s">
         <v>196</v>
@@ -5011,66 +5099,66 @@
     </row>
     <row r="45" spans="1:5" ht="18.600000000000001" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="C45" s="33">
         <v>98</v>
       </c>
       <c r="D45" s="24" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17.45" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C46" s="49">
         <v>98</v>
       </c>
       <c r="D46" s="24" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.95">
       <c r="A47" s="8" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="C47" s="23">
         <v>90</v>
       </c>
       <c r="D47" s="57" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="E47" t="s">
-        <v>270</v>
+        <v>203</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="15.95">
       <c r="A48" s="2" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="C48" s="23">
         <v>98</v>
       </c>
       <c r="D48" s="59" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.95">
       <c r="A49" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="23"/>
@@ -5078,38 +5166,38 @@
     </row>
     <row r="50" spans="1:4" ht="15.95">
       <c r="A50" s="8" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="C50" s="23">
         <v>99</v>
       </c>
       <c r="D50" s="24" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A51" s="8" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C51" s="32">
         <v>98</v>
       </c>
       <c r="D51" s="24" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15.6" customHeight="1">
       <c r="A52" s="8" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="C52" s="23">
         <v>99</v>
@@ -5118,133 +5206,147 @@
     </row>
     <row r="53" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A53" s="8" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="C53" s="31">
         <v>99</v>
       </c>
       <c r="D53" s="24" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.95">
       <c r="A54" s="18" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="C54" s="23">
         <v>98</v>
       </c>
       <c r="D54" s="59" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15.95">
       <c r="A55" s="19" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="C55" s="23">
         <v>98</v>
       </c>
       <c r="D55" s="59" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="17.100000000000001" customHeight="1">
       <c r="A56" s="19" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="C56" s="23">
         <v>99</v>
       </c>
       <c r="D56" s="59" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15.95">
       <c r="A57" s="9" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C57" s="23">
         <v>98</v>
       </c>
       <c r="D57" s="24" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="58"/>
-      <c r="D58" s="55"/>
+      <c r="D58" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="59" spans="1:4" ht="30" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="23"/>
-      <c r="D59" s="57"/>
+      <c r="D59" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="60" spans="1:4" ht="19.5" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="23"/>
-      <c r="D60" s="57"/>
+      <c r="D60" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="61" spans="1:4" ht="18.75" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="23"/>
-      <c r="D61" s="57"/>
+      <c r="D61" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="62" spans="1:4" ht="17.45" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="32"/>
-      <c r="D62" s="57"/>
+      <c r="D62" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="63" spans="1:4" ht="18" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="23"/>
-      <c r="D63" s="57"/>
+      <c r="D63" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="64" spans="1:4" ht="18" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="53"/>
-      <c r="D64" s="57"/>
+      <c r="D64" s="70" t="s">
+        <v>301</v>
+      </c>
     </row>
     <row r="65" spans="1:4" ht="32.25" customHeight="1">
       <c r="A65" s="3" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="52"/>
@@ -5252,10 +5354,10 @@
     </row>
     <row r="66" spans="1:4" ht="18" customHeight="1">
       <c r="A66" s="28" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C66" s="30" t="s">
         <v>197</v>
@@ -5264,7 +5366,7 @@
     </row>
     <row r="67" spans="1:4" ht="15.95">
       <c r="A67" s="2" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B67" s="24"/>
       <c r="C67" s="10"/>
@@ -5272,7 +5374,7 @@
     </row>
     <row r="68" spans="1:4" ht="15.95">
       <c r="A68" s="2" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B68" s="24"/>
       <c r="C68" s="10"/>
@@ -5280,7 +5382,7 @@
     </row>
     <row r="69" spans="1:4" ht="15.95">
       <c r="A69" s="2" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="B69" s="24"/>
       <c r="C69" s="10"/>
@@ -5288,7 +5390,7 @@
     </row>
     <row r="70" spans="1:4" ht="15.95">
       <c r="A70" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="B70" s="24"/>
       <c r="C70" s="10"/>
@@ -5296,7 +5398,7 @@
     </row>
     <row r="71" spans="1:4" ht="15.95">
       <c r="A71" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B71" s="24"/>
       <c r="C71" s="10"/>
@@ -5304,7 +5406,7 @@
     </row>
     <row r="72" spans="1:4" ht="15.95">
       <c r="A72" s="2" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B72" s="24"/>
       <c r="C72" s="10"/>
@@ -5312,7 +5414,7 @@
     </row>
     <row r="73" spans="1:4" ht="15.95">
       <c r="A73" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B73" s="24"/>
       <c r="C73" s="10"/>
@@ -5320,7 +5422,7 @@
     </row>
     <row r="74" spans="1:4" ht="15.95">
       <c r="A74" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="B74" s="24"/>
       <c r="C74" s="10"/>
@@ -5328,7 +5430,7 @@
     </row>
     <row r="75" spans="1:4" ht="15.95">
       <c r="A75" s="2" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B75" s="24"/>
       <c r="C75" s="10"/>
@@ -5336,7 +5438,7 @@
     </row>
     <row r="76" spans="1:4" ht="15.95">
       <c r="A76" s="2" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="B76" s="24"/>
       <c r="C76" s="10"/>
@@ -5344,7 +5446,7 @@
     </row>
     <row r="77" spans="1:4" ht="15.95">
       <c r="A77" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B77" s="24"/>
       <c r="C77" s="10"/>
@@ -5352,7 +5454,7 @@
     </row>
     <row r="78" spans="1:4" ht="15.95">
       <c r="A78" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B78" s="24"/>
       <c r="C78" s="10"/>
@@ -5360,7 +5462,7 @@
     </row>
     <row r="79" spans="1:4" ht="15.95">
       <c r="A79" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B79" s="24"/>
       <c r="C79" s="10"/>
@@ -5368,7 +5470,7 @@
     </row>
     <row r="80" spans="1:4" ht="15.95">
       <c r="A80" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B80" s="33"/>
       <c r="C80" s="23"/>
@@ -5376,7 +5478,7 @@
     </row>
     <row r="81" spans="1:4" ht="15.95">
       <c r="A81" s="43" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B81" s="24"/>
       <c r="C81" s="32"/>
@@ -5384,7 +5486,7 @@
     </row>
     <row r="82" spans="1:4" ht="15.95">
       <c r="A82" s="51" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B82" s="24"/>
       <c r="C82" s="32"/>
@@ -5392,7 +5494,7 @@
     </row>
     <row r="83" spans="1:4" ht="15.95">
       <c r="A83" s="22" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="B83" s="33"/>
       <c r="C83" s="23"/>
@@ -5400,7 +5502,7 @@
     </row>
     <row r="84" spans="1:4" ht="15.95">
       <c r="A84" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B84" s="24"/>
       <c r="C84" s="10"/>
@@ -5408,7 +5510,7 @@
     </row>
     <row r="85" spans="1:4" ht="15.95">
       <c r="A85" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B85" s="24"/>
       <c r="C85" s="10"/>
@@ -5416,7 +5518,7 @@
     </row>
     <row r="86" spans="1:4" ht="15.95">
       <c r="A86" s="2" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B86" s="10"/>
       <c r="C86" s="10"/>
@@ -5424,7 +5526,7 @@
     </row>
     <row r="87" spans="1:4" ht="15.95">
       <c r="A87" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B87" s="10"/>
       <c r="C87" s="10"/>
@@ -5432,7 +5534,7 @@
     </row>
     <row r="88" spans="1:4" ht="15.95">
       <c r="A88" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B88" s="24"/>
       <c r="C88" s="10"/>
@@ -5440,7 +5542,7 @@
     </row>
     <row r="89" spans="1:4" ht="15.95">
       <c r="A89" s="2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B89" s="24"/>
       <c r="C89" s="10"/>
@@ -5448,7 +5550,7 @@
     </row>
     <row r="90" spans="1:4" ht="15.95">
       <c r="A90" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B90" s="24"/>
       <c r="C90" s="10"/>
@@ -5456,7 +5558,7 @@
     </row>
     <row r="91" spans="1:4" ht="15.95">
       <c r="A91" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="B91" s="10">
         <v>80000</v>
@@ -5470,7 +5572,7 @@
     </row>
     <row r="92" spans="1:4" ht="15.95">
       <c r="A92" s="2" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="B92" s="24">
         <v>80000</v>
@@ -5484,19 +5586,19 @@
     </row>
     <row r="93" spans="1:4" ht="15.95">
       <c r="A93" s="2" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B93" s="70">
         <v>51000</v>
       </c>
       <c r="C93" s="57"/>
       <c r="D93" s="71" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.95">
       <c r="A94" s="2" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="B94" s="24">
         <v>32000</v>
@@ -5510,7 +5612,7 @@
     </row>
     <row r="95" spans="1:4" ht="15.95">
       <c r="A95" s="2" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="B95" s="24">
         <v>32000</v>
@@ -5524,43 +5626,61 @@
     </row>
     <row r="96" spans="1:4" ht="15.95">
       <c r="A96" s="8" t="s">
-        <v>334</v>
-      </c>
-      <c r="B96" s="34"/>
-      <c r="C96" s="35"/>
-      <c r="D96" s="10"/>
+        <v>341</v>
+      </c>
+      <c r="B96" s="34">
+        <v>8000</v>
+      </c>
+      <c r="C96" s="35">
+        <v>74</v>
+      </c>
+      <c r="D96" s="10">
+        <v>48</v>
+      </c>
     </row>
     <row r="97" spans="1:10" ht="15.95">
       <c r="A97" s="2" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="B97" s="72">
         <v>26000</v>
       </c>
       <c r="C97" s="70"/>
       <c r="D97" s="70" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
     </row>
     <row r="98" spans="1:10" ht="15.95">
       <c r="A98" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="B98" s="72"/>
-      <c r="C98" s="70"/>
-      <c r="D98" s="70"/>
+        <v>344</v>
+      </c>
+      <c r="B98" s="24">
+        <v>1000</v>
+      </c>
+      <c r="C98" s="24">
+        <v>99</v>
+      </c>
+      <c r="D98" s="24">
+        <v>57</v>
+      </c>
     </row>
     <row r="99" spans="1:10" ht="15.95">
       <c r="A99" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="B99" s="24"/>
-      <c r="C99" s="10"/>
-      <c r="D99" s="10"/>
+        <v>345</v>
+      </c>
+      <c r="B99" s="24">
+        <v>300</v>
+      </c>
+      <c r="C99" s="10">
+        <v>99</v>
+      </c>
+      <c r="D99" s="10">
+        <v>69</v>
+      </c>
     </row>
     <row r="100" spans="1:10" ht="15.95">
       <c r="A100" s="2" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="B100" s="16"/>
       <c r="C100" s="10"/>
@@ -5568,7 +5688,7 @@
     </row>
     <row r="101" spans="1:10" ht="15.95">
       <c r="A101" s="2" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B101" s="10"/>
       <c r="C101" s="10"/>
@@ -5576,7 +5696,7 @@
     </row>
     <row r="102" spans="1:10" ht="15.95">
       <c r="A102" s="2" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="B102" s="24"/>
       <c r="C102" s="10"/>
@@ -5613,7 +5733,7 @@
   <cols>
     <col min="1" max="1" width="87.85546875" customWidth="1"/>
     <col min="2" max="2" width="19.42578125" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="22.140625" style="5" customWidth="1"/>
     <col min="4" max="4" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
     <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
@@ -5621,10 +5741,10 @@
   <sheetData>
     <row r="1" spans="1:5" ht="57" customHeight="1">
       <c r="A1" s="50" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="C1" s="36" t="s">
         <v>194</v>
@@ -5650,7 +5770,7 @@
         <v>199</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="C3" s="59">
         <v>91</v>
@@ -5664,7 +5784,7 @@
         <v>201</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C4" s="4">
         <v>70</v>
@@ -5673,12 +5793,12 @@
         <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.6" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B5" s="4"/>
       <c r="C5" s="4"/>
@@ -5686,10 +5806,10 @@
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="C6" s="4">
         <v>94</v>
@@ -5700,10 +5820,10 @@
     </row>
     <row r="7" spans="1:5" ht="14.45" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="C7" s="59">
         <v>96</v>
@@ -5714,10 +5834,10 @@
     </row>
     <row r="8" spans="1:5" ht="14.1" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="C8" s="4">
         <v>90</v>
@@ -5726,12 +5846,12 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" ht="15.95">
       <c r="A9" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="C9" s="59">
         <v>90</v>
@@ -5740,12 +5860,12 @@
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" ht="15.95">
       <c r="A10" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="C10" s="4">
         <v>90</v>
@@ -5756,26 +5876,26 @@
     </row>
     <row r="11" spans="1:5" ht="15.95">
       <c r="A11" s="2" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="59"/>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" ht="15.95">
       <c r="A12" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="59"/>
       <c r="D12" s="59"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" ht="15.95">
       <c r="A13" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
       <c r="C13" s="4">
         <v>90</v>
@@ -5784,12 +5904,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" ht="15.95">
       <c r="A14" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>353</v>
+        <v>360</v>
       </c>
       <c r="C14" s="4">
         <v>90</v>
@@ -5798,12 +5918,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" ht="15.95">
       <c r="A15" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>354</v>
+        <v>361</v>
       </c>
       <c r="C15" s="4">
         <v>94</v>
@@ -5814,7 +5934,7 @@
     </row>
     <row r="16" spans="1:5" ht="15.95">
       <c r="A16" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B16" s="46"/>
       <c r="C16" s="4"/>
@@ -5822,7 +5942,7 @@
     </row>
     <row r="17" spans="1:6" ht="15.95">
       <c r="A17" s="43" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
@@ -5830,10 +5950,10 @@
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1">
       <c r="A18" s="38" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>197</v>
@@ -5844,10 +5964,10 @@
     </row>
     <row r="19" spans="1:6" ht="15.95">
       <c r="A19" s="22" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="C19" s="55">
         <v>92</v>
@@ -5858,10 +5978,10 @@
     </row>
     <row r="20" spans="1:6" ht="15.95">
       <c r="A20" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="C20" s="57">
         <v>95</v>
@@ -5872,7 +5992,7 @@
     </row>
     <row r="21" spans="1:6" ht="15.95">
       <c r="A21" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B21" s="10"/>
       <c r="C21" s="57"/>
@@ -5880,10 +6000,10 @@
     </row>
     <row r="22" spans="1:6" ht="15.95">
       <c r="A22" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="C22" s="57">
         <v>93</v>
@@ -5894,10 +6014,10 @@
     </row>
     <row r="23" spans="1:6" ht="15.95">
       <c r="A23" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>359</v>
+        <v>366</v>
       </c>
       <c r="C23" s="57">
         <v>92</v>
@@ -5906,12 +6026,12 @@
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" ht="15.95">
       <c r="A24" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="C24" s="57">
         <v>92</v>
@@ -5920,15 +6040,15 @@
         <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="15.95">
       <c r="A25" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="C25" s="57">
         <v>92</v>
@@ -5937,12 +6057,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" ht="15.95">
       <c r="A26" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>360</v>
+        <v>367</v>
       </c>
       <c r="C26" s="57">
         <v>90</v>
@@ -5951,12 +6071,12 @@
         <v>69</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" ht="15.95">
       <c r="A27" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="C27" s="57">
         <v>90</v>
@@ -5965,12 +6085,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" ht="15.95">
       <c r="A28" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="C28" s="57">
         <v>92</v>
@@ -5981,10 +6101,10 @@
     </row>
     <row r="29" spans="1:6" ht="18" customHeight="1">
       <c r="A29" s="29" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>197</v>
@@ -5995,7 +6115,7 @@
     </row>
     <row r="30" spans="1:6" ht="15.95">
       <c r="A30" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B30" s="47"/>
       <c r="C30" s="57"/>
@@ -6003,7 +6123,7 @@
     </row>
     <row r="31" spans="1:6" ht="15.95">
       <c r="A31" s="2" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B31" s="47"/>
       <c r="C31" s="57"/>
@@ -6011,7 +6131,7 @@
     </row>
     <row r="32" spans="1:6" ht="15.95">
       <c r="A32" s="2" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="B32" s="47"/>
       <c r="C32" s="57"/>
@@ -6019,7 +6139,7 @@
     </row>
     <row r="33" spans="1:4" ht="17.45" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B33" s="47"/>
       <c r="C33" s="54"/>
@@ -6027,10 +6147,10 @@
     </row>
     <row r="34" spans="1:4" ht="18" customHeight="1">
       <c r="A34" s="29" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="C34" s="40" t="s">
         <v>197</v>
@@ -6041,7 +6161,7 @@
     </row>
     <row r="35" spans="1:4" ht="15.95">
       <c r="A35" s="2" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B35" s="48">
         <v>26000</v>
@@ -6055,7 +6175,7 @@
     </row>
     <row r="36" spans="1:4" ht="15.95">
       <c r="A36" s="2" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B36" s="4">
         <v>25400</v>
@@ -6069,7 +6189,7 @@
     </row>
     <row r="37" spans="1:4" ht="15.6" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B37" s="4">
         <v>13300</v>
@@ -6083,7 +6203,7 @@
     </row>
     <row r="38" spans="1:4" ht="15.95">
       <c r="A38" s="2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B38" s="4">
         <v>3200</v>
@@ -6095,9 +6215,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:4">
+    <row r="39" spans="1:4" ht="15.95">
       <c r="A39" s="22" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B39" s="15">
         <v>2700</v>
@@ -6111,7 +6231,7 @@
     </row>
     <row r="40" spans="1:4" ht="15.95">
       <c r="A40" s="22" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B40" s="45"/>
       <c r="C40" s="15"/>
@@ -6119,13 +6239,13 @@
     </row>
     <row r="41" spans="1:4" ht="15.95">
       <c r="A41" s="2" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B41" s="4">
         <v>1810</v>
       </c>
-      <c r="C41" s="4">
-        <v>95</v>
+      <c r="C41" s="4" t="s">
+        <v>373</v>
       </c>
       <c r="D41" s="59">
         <v>68</v>
@@ -6133,7 +6253,7 @@
     </row>
     <row r="42" spans="1:4" ht="15.95">
       <c r="A42" s="2" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B42" s="1">
         <v>460</v>
@@ -6147,7 +6267,7 @@
     </row>
     <row r="43" spans="1:4" ht="15.95">
       <c r="A43" s="2" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B43" s="4"/>
       <c r="C43" s="4"/>
@@ -6155,77 +6275,77 @@
     </row>
     <row r="44" spans="1:4" ht="18" customHeight="1">
       <c r="A44" s="29" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C44" s="40" t="s">
         <v>197</v>
       </c>
       <c r="D44" s="40" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="18.600000000000001" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="C45" s="24">
         <v>98</v>
       </c>
       <c r="D45" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="17.45" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B46" s="49" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C46" s="24">
         <v>98</v>
       </c>
       <c r="D46" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.95">
       <c r="A47" s="8" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="C47" s="57">
         <v>96</v>
       </c>
       <c r="D47" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.95">
       <c r="A48" s="2" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="B48" s="49" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C48" s="57">
         <v>96</v>
       </c>
       <c r="D48" s="59" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.95">
       <c r="A49" s="2" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B49" s="23"/>
       <c r="C49" s="57"/>
@@ -6233,119 +6353,119 @@
     </row>
     <row r="50" spans="1:4" ht="15.95">
       <c r="A50" s="8" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="C50" s="55">
         <v>98</v>
       </c>
       <c r="D50" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A51" s="8" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B51" s="32" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C51" s="57">
         <v>98</v>
       </c>
       <c r="D51" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15.6" customHeight="1">
       <c r="A52" s="8" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="B52" s="58" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="C52" s="57">
         <v>99</v>
       </c>
       <c r="D52" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A53" s="8" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="B53" s="31" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="C53" s="65">
         <v>99</v>
       </c>
       <c r="D53" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.95">
       <c r="A54" s="18" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="B54" s="23" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="C54" s="66">
         <v>98</v>
       </c>
       <c r="D54" s="59" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15.95">
       <c r="A55" s="19" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="B55" s="23" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="C55" s="66">
         <v>98</v>
       </c>
       <c r="D55" s="59" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="17.100000000000001" customHeight="1">
       <c r="A56" s="19" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C56" s="66">
         <v>96</v>
       </c>
       <c r="D56" s="59" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15.95">
       <c r="A57" s="9" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B57" s="25" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="C57" s="57">
         <v>96</v>
       </c>
       <c r="D57" s="59" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="B58" s="23"/>
       <c r="C58" s="55"/>
@@ -6353,7 +6473,7 @@
     </row>
     <row r="59" spans="1:4" ht="30" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="B59" s="23"/>
       <c r="C59" s="57"/>
@@ -6361,7 +6481,7 @@
     </row>
     <row r="60" spans="1:4" ht="19.5" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="B60" s="23"/>
       <c r="C60" s="57"/>
@@ -6369,7 +6489,7 @@
     </row>
     <row r="61" spans="1:4" ht="18.75" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B61" s="23"/>
       <c r="C61" s="57"/>
@@ -6377,7 +6497,7 @@
     </row>
     <row r="62" spans="1:4" ht="17.45" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="B62" s="32"/>
       <c r="C62" s="57"/>
@@ -6385,7 +6505,7 @@
     </row>
     <row r="63" spans="1:4" ht="18" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B63" s="23"/>
       <c r="C63" s="57"/>
@@ -6393,7 +6513,7 @@
     </row>
     <row r="64" spans="1:4" ht="18" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="B64" s="53"/>
       <c r="C64" s="57"/>
@@ -6401,7 +6521,7 @@
     </row>
     <row r="65" spans="1:4" ht="32.25" customHeight="1">
       <c r="A65" s="3" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="B65" s="52"/>
       <c r="C65" s="57"/>
@@ -6409,21 +6529,21 @@
     </row>
     <row r="66" spans="1:4" ht="18" customHeight="1">
       <c r="A66" s="28" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B66" s="30" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C66" s="67" t="s">
         <v>197</v>
       </c>
       <c r="D66" s="67" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="15.95">
       <c r="A67" s="2" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="B67" s="10"/>
       <c r="C67" s="57"/>
@@ -6431,7 +6551,7 @@
     </row>
     <row r="68" spans="1:4" ht="15.95">
       <c r="A68" s="2" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B68" s="10"/>
       <c r="C68" s="57"/>
@@ -6439,7 +6559,7 @@
     </row>
     <row r="69" spans="1:4" ht="15.95">
       <c r="A69" s="2" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="B69" s="10"/>
       <c r="C69" s="57"/>
@@ -6447,7 +6567,7 @@
     </row>
     <row r="70" spans="1:4" ht="15.95">
       <c r="A70" s="2" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="B70" s="10"/>
       <c r="C70" s="57"/>
@@ -6455,7 +6575,7 @@
     </row>
     <row r="71" spans="1:4" ht="15.95">
       <c r="A71" s="2" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B71" s="10"/>
       <c r="C71" s="57"/>
@@ -6463,7 +6583,7 @@
     </row>
     <row r="72" spans="1:4" ht="15.95">
       <c r="A72" s="2" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B72" s="10"/>
       <c r="C72" s="57"/>
@@ -6471,7 +6591,7 @@
     </row>
     <row r="73" spans="1:4" ht="15.95">
       <c r="A73" s="2" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="B73" s="10"/>
       <c r="C73" s="57"/>
@@ -6479,7 +6599,7 @@
     </row>
     <row r="74" spans="1:4" ht="15.95">
       <c r="A74" s="2" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="B74" s="10">
         <v>1536</v>
@@ -6489,7 +6609,7 @@
     </row>
     <row r="75" spans="1:4" ht="15.95">
       <c r="A75" s="2" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B75" s="10"/>
       <c r="C75" s="57"/>
@@ -6497,7 +6617,7 @@
     </row>
     <row r="76" spans="1:4" ht="15.95">
       <c r="A76" s="2" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="B76" s="10"/>
       <c r="C76" s="57"/>
@@ -6505,7 +6625,7 @@
     </row>
     <row r="77" spans="1:4" ht="15.95">
       <c r="A77" s="2" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="B77" s="10"/>
       <c r="C77" s="57"/>
@@ -6513,7 +6633,7 @@
     </row>
     <row r="78" spans="1:4" ht="15.95">
       <c r="A78" s="2" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B78" s="10"/>
       <c r="C78" s="57"/>
@@ -6521,7 +6641,7 @@
     </row>
     <row r="79" spans="1:4" ht="15.95">
       <c r="A79" s="2" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="B79" s="10"/>
       <c r="C79" s="57"/>
@@ -6529,7 +6649,7 @@
     </row>
     <row r="80" spans="1:4" ht="15.95">
       <c r="A80" s="2" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="B80" s="23"/>
       <c r="C80" s="57"/>
@@ -6537,7 +6657,7 @@
     </row>
     <row r="81" spans="1:4" ht="15.95">
       <c r="A81" s="43" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B81" s="32"/>
       <c r="C81" s="57"/>
@@ -6545,7 +6665,7 @@
     </row>
     <row r="82" spans="1:4" ht="15.95">
       <c r="A82" s="51" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="B82" s="32"/>
       <c r="C82" s="57"/>
@@ -6553,7 +6673,7 @@
     </row>
     <row r="83" spans="1:4" ht="15.95">
       <c r="A83" s="22" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="B83" s="23"/>
       <c r="C83" s="57"/>
@@ -6561,7 +6681,7 @@
     </row>
     <row r="84" spans="1:4" ht="15.95">
       <c r="A84" s="2" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B84" s="10"/>
       <c r="C84" s="57"/>
@@ -6569,7 +6689,7 @@
     </row>
     <row r="85" spans="1:4" ht="15.95">
       <c r="A85" s="2" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="B85" s="10"/>
       <c r="C85" s="57"/>
@@ -6577,27 +6697,27 @@
     </row>
     <row r="86" spans="1:4" ht="15.95">
       <c r="A86" s="2" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="C86" s="71"/>
       <c r="D86" s="71"/>
     </row>
     <row r="87" spans="1:4" ht="15.95">
       <c r="A87" s="2" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="C87" s="71"/>
       <c r="D87" s="71"/>
     </row>
     <row r="88" spans="1:4" ht="15.95">
       <c r="A88" s="2" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="B88" s="10"/>
       <c r="C88" s="57"/>
@@ -6605,7 +6725,7 @@
     </row>
     <row r="89" spans="1:4" ht="15.95">
       <c r="A89" s="2" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="B89" s="10"/>
       <c r="C89" s="57"/>
@@ -6613,7 +6733,7 @@
     </row>
     <row r="90" spans="1:4" ht="15.95">
       <c r="A90" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B90" s="10"/>
       <c r="C90" s="57"/>
@@ -6621,7 +6741,7 @@
     </row>
     <row r="91" spans="1:4" ht="15.95">
       <c r="A91" s="2" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="B91" s="10">
         <v>96000</v>
@@ -6635,7 +6755,7 @@
     </row>
     <row r="92" spans="1:4" ht="15.95">
       <c r="A92" s="2" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="B92" s="10">
         <v>96000</v>
@@ -6649,19 +6769,19 @@
     </row>
     <row r="93" spans="1:4" ht="15.95">
       <c r="A93" s="2" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B93" s="70">
         <v>51000</v>
       </c>
       <c r="C93" s="57"/>
       <c r="D93" s="71" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.95">
       <c r="A94" s="2" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="B94" s="73"/>
       <c r="C94" s="56"/>
@@ -6669,7 +6789,7 @@
     </row>
     <row r="95" spans="1:4" ht="15.95">
       <c r="A95" s="2" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="B95" s="26"/>
       <c r="C95" s="56"/>
@@ -6677,7 +6797,7 @@
     </row>
     <row r="96" spans="1:4" ht="15.95">
       <c r="A96" s="8" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="B96" s="35"/>
       <c r="C96" s="10"/>
@@ -6685,7 +6805,7 @@
     </row>
     <row r="97" spans="1:9" ht="15.95">
       <c r="A97" s="2" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="B97" s="10"/>
       <c r="C97" s="10"/>
@@ -6693,7 +6813,7 @@
     </row>
     <row r="98" spans="1:9" ht="15.95">
       <c r="A98" s="2" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="B98" s="10">
         <v>1200</v>
@@ -6707,7 +6827,7 @@
     </row>
     <row r="99" spans="1:9" ht="15.95">
       <c r="A99" s="2" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="B99" s="10"/>
       <c r="C99" s="10"/>
@@ -6715,7 +6835,7 @@
     </row>
     <row r="100" spans="1:9" ht="15.95">
       <c r="A100" s="2" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="B100" s="10"/>
       <c r="C100" s="10"/>
@@ -6723,7 +6843,7 @@
     </row>
     <row r="101" spans="1:9" ht="15.95">
       <c r="A101" s="2" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B101" s="10"/>
       <c r="C101" s="10"/>
@@ -6731,7 +6851,7 @@
     </row>
     <row r="102" spans="1:9" ht="15.95">
       <c r="A102" s="2" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="B102" s="10"/>
       <c r="C102" s="10"/>
@@ -6771,10 +6891,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="60">
       <c r="A1" s="50" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="C1" s="36" t="s">
         <v>194</v>
@@ -6785,346 +6905,346 @@
         <v>195</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="C2" s="40"/>
     </row>
     <row r="3" spans="1:3" ht="18.95" hidden="1">
       <c r="A3" s="22" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="42"/>
     </row>
     <row r="4" spans="1:3" ht="15.95" hidden="1">
       <c r="A4" s="2" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="15.95" hidden="1">
       <c r="A5" s="2" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="59"/>
     </row>
     <row r="6" spans="1:3" ht="15.95" hidden="1">
       <c r="A6" s="2" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
     </row>
     <row r="7" spans="1:3" ht="15.95" hidden="1">
       <c r="A7" s="2" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
     </row>
     <row r="8" spans="1:3" ht="15.95">
       <c r="A8" s="2" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="C8" s="60" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.95">
       <c r="A9" s="2" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C9" s="59" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.95" hidden="1">
       <c r="A10" s="2" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
     </row>
     <row r="11" spans="1:3" ht="15.95" hidden="1">
       <c r="A11" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="59"/>
     </row>
     <row r="12" spans="1:3" ht="15.95" hidden="1">
       <c r="A12" s="2" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
     </row>
     <row r="13" spans="1:3" ht="15.95" hidden="1">
       <c r="A13" s="2" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="59"/>
     </row>
     <row r="14" spans="1:3" ht="15.95" hidden="1">
       <c r="A14" s="2" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" ht="15.95" hidden="1">
       <c r="A15" s="2" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
     </row>
     <row r="16" spans="1:3" ht="15.95" hidden="1">
       <c r="A16" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="4"/>
     </row>
     <row r="17" spans="1:3" ht="15.95" hidden="1">
       <c r="A17" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" ht="15.95" hidden="1">
       <c r="A18" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="4"/>
     </row>
     <row r="19" spans="1:3" ht="15.95" hidden="1">
       <c r="A19" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B19" s="46"/>
       <c r="C19" s="4"/>
     </row>
     <row r="20" spans="1:3" ht="15.95" hidden="1">
       <c r="A20" s="43" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
     </row>
     <row r="21" spans="1:3" ht="18.95">
       <c r="A21" s="38" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B21" s="40"/>
       <c r="C21" s="61"/>
     </row>
     <row r="22" spans="1:3" ht="15.95" hidden="1">
       <c r="A22" s="22" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B22" s="27"/>
       <c r="C22" s="55"/>
     </row>
     <row r="23" spans="1:3" ht="15.95">
       <c r="A23" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.95" hidden="1">
       <c r="A24" s="2" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B24" s="10"/>
       <c r="C24" s="57"/>
     </row>
     <row r="25" spans="1:3" ht="15.95">
       <c r="A25" s="2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.95">
       <c r="A26" s="2" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="C26" s="57" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.95" hidden="1">
       <c r="A27" s="2" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="57"/>
     </row>
     <row r="28" spans="1:3" ht="15.95" hidden="1">
       <c r="A28" s="2" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="B28" s="10"/>
       <c r="C28" s="57"/>
     </row>
     <row r="29" spans="1:3" ht="15.95" hidden="1">
       <c r="A29" s="2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="B29" s="10"/>
       <c r="C29" s="57"/>
     </row>
     <row r="30" spans="1:3" ht="15.95" hidden="1">
       <c r="A30" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="57"/>
     </row>
     <row r="31" spans="1:3" ht="15.95" hidden="1">
       <c r="A31" s="2" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="B31" s="10"/>
       <c r="C31" s="57"/>
     </row>
     <row r="32" spans="1:3" ht="18.95" hidden="1">
       <c r="A32" s="29" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
       <c r="B32" s="14"/>
       <c r="C32" s="62"/>
     </row>
     <row r="33" spans="1:3" ht="15.95" hidden="1">
       <c r="A33" s="2" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="B33" s="47"/>
       <c r="C33" s="57"/>
     </row>
     <row r="34" spans="1:3" ht="15.95" hidden="1">
       <c r="A34" s="2" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="B34" s="47"/>
       <c r="C34" s="57"/>
     </row>
     <row r="35" spans="1:3" ht="15.95" hidden="1">
       <c r="A35" s="2" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="B35" s="47"/>
       <c r="C35" s="57"/>
     </row>
     <row r="36" spans="1:3" ht="15.95" hidden="1">
       <c r="A36" s="2" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B36" s="47"/>
       <c r="C36" s="54"/>
     </row>
     <row r="37" spans="1:3" ht="18.95">
       <c r="A37" s="29" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B37" s="12"/>
       <c r="C37" s="63"/>
     </row>
     <row r="38" spans="1:3" ht="15.95" hidden="1">
       <c r="A38" s="2" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B38" s="48"/>
       <c r="C38" s="64"/>
     </row>
     <row r="39" spans="1:3" ht="15.95" hidden="1">
       <c r="A39" s="2" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="64"/>
     </row>
     <row r="40" spans="1:3" ht="15.95">
       <c r="A40" s="2" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="C40" s="60" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.95">
       <c r="A41" s="2" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="C41" s="60" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.95" hidden="1">
       <c r="A42" s="22" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
     </row>
     <row r="43" spans="1:3" ht="15.95" hidden="1">
       <c r="A43" s="22" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B43" s="45"/>
       <c r="C43" s="15"/>
     </row>
     <row r="44" spans="1:3" ht="15.95" hidden="1">
       <c r="A44" s="2" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
     </row>
     <row r="45" spans="1:3" ht="15.95">
       <c r="A45" s="2" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15.95" hidden="1">
       <c r="A46" s="2" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -7135,6 +7255,118 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9bf4d24f-a117-48f7-91e1-2035a8c734fd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="cb645b5b-9a36-43da-96bf-ab72ec91ddff" xsi:nil="true"/>
+    <SharedWithUsers xmlns="0b7692b1-2532-40e4-a300-4d7fced4a07a">
+      <UserInfo>
+        <DisplayName>Anand Thulasiram</DisplayName>
+        <AccountId>2178</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Vipin Kumar</DisplayName>
+        <AccountId>64</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Sunil  Masineni</DisplayName>
+        <AccountId>5184</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Geetha B K</DisplayName>
+        <AccountId>63</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Jagadeesh Rajashekharaiah</DisplayName>
+        <AccountId>13</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Deepasri Chittala</DisplayName>
+        <AccountId>4801</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Weibin Chen</DisplayName>
+        <AccountId>317</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Xiaochen Tang</DisplayName>
+        <AccountId>910</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Anand Antur</DisplayName>
+        <AccountId>670</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Venu Maya</DisplayName>
+        <AccountId>33</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Chockalingam Balasubramanian</DisplayName>
+        <AccountId>682</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Neetu Rathee</DisplayName>
+        <AccountId>4709</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Prasad Shroff</DisplayName>
+        <AccountId>4142</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Kedar Dhuru</DisplayName>
+        <AccountId>3907</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Sarvesh Batta</DisplayName>
+        <AccountId>21</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Shankar Satyamurthy</DisplayName>
+        <AccountId>3116</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>David Passamonte</DisplayName>
+        <AccountId>5189</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="a3ce5a06-b323-45b4-8d97-2f59321c9a5a" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010092711BC64AAEC84E9EF800276F1AD52C" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba397f1440615f1339f1f20b24e67478">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9bf4d24f-a117-48f7-91e1-2035a8c734fd" xmlns:ns3="0b7692b1-2532-40e4-a300-4d7fced4a07a" xmlns:ns4="cb645b5b-9a36-43da-96bf-ab72ec91ddff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="74828cee37efa74eab9b700f6a6651cc" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="9bf4d24f-a117-48f7-91e1-2035a8c734fd"/>
@@ -7382,130 +7614,18 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9bf4d24f-a117-48f7-91e1-2035a8c734fd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="cb645b5b-9a36-43da-96bf-ab72ec91ddff" xsi:nil="true"/>
-    <SharedWithUsers xmlns="0b7692b1-2532-40e4-a300-4d7fced4a07a">
-      <UserInfo>
-        <DisplayName>Anand Thulasiram</DisplayName>
-        <AccountId>2178</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Vipin Kumar</DisplayName>
-        <AccountId>64</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Sunil  Masineni</DisplayName>
-        <AccountId>5184</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Geetha B K</DisplayName>
-        <AccountId>63</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Jagadeesh Rajashekharaiah</DisplayName>
-        <AccountId>13</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Deepasri Chittala</DisplayName>
-        <AccountId>4801</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Weibin Chen</DisplayName>
-        <AccountId>317</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Xiaochen Tang</DisplayName>
-        <AccountId>910</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Anand Antur</DisplayName>
-        <AccountId>670</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Venu Maya</DisplayName>
-        <AccountId>33</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Chockalingam Balasubramanian</DisplayName>
-        <AccountId>682</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Neetu Rathee</DisplayName>
-        <AccountId>4709</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Prasad Shroff</DisplayName>
-        <AccountId>4142</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Kedar Dhuru</DisplayName>
-        <AccountId>3907</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Sarvesh Batta</DisplayName>
-        <AccountId>21</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Shankar Satyamurthy</DisplayName>
-        <AccountId>3116</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>David Passamonte</DisplayName>
-        <AccountId>5189</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="a3ce5a06-b323-45b4-8d97-2f59321c9a5a" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C639165A-13FF-4A9F-A5E9-0E8F0976D502}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3D764E2-0E35-4957-B738-9033D3F0B0F5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3D764E2-0E35-4957-B738-9033D3F0B0F5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D75EC423-2542-4A93-99FE-CC28AA840E8C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D75EC423-2542-4A93-99FE-CC28AA840E8C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CF876B3-44D4-4080-B40E-3DF67289D40E}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CF876B3-44D4-4080-B40E-3DF67289D40E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C639165A-13FF-4A9F-A5E9-0E8F0976D502}"/>
 </file>
</xml_diff>

<commit_message>
Add dual-axis vertical grouped bar chart with automatic Daily Sanity data visualization
</commit_message>
<xml_diff>
--- a/public/data/SRX4XX_Datasheet.xlsx
+++ b/public/data/SRX4XX_Datasheet.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30117"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30126"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpe-my.sharepoint.com/personal/antony-ruban_alexis_hpe_com/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="507" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FE324C9-AB4A-45FE-80DA-F616BB142F87}"/>
+  <xr:revisionPtr revIDLastSave="637" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39540F41-77DD-4392-B620-9ED377082040}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="20140" firstSheet="1" activeTab="2" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
+    <workbookView xWindow="1200" yWindow="600" windowWidth="36000" windowHeight="19740" firstSheet="2" activeTab="3" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
   </bookViews>
   <sheets>
     <sheet name="ISSUES-PR's" sheetId="7" r:id="rId1"/>
     <sheet name="SRX400" sheetId="6" r:id="rId2"/>
     <sheet name="SRX440" sheetId="10" r:id="rId3"/>
-    <sheet name="Prelimnary data" sheetId="9" r:id="rId4"/>
-    <sheet name="Second Set Data" sheetId="11" r:id="rId5"/>
+    <sheet name="DS-1" sheetId="12" r:id="rId4"/>
+    <sheet name="Prelimnary data" sheetId="9" r:id="rId5"/>
+    <sheet name="Second Set Data" sheetId="11" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ISSUES-PR''s'!$A$1:$H$94</definedName>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1124" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="466">
   <si>
     <t>number</t>
   </si>
@@ -830,10 +831,13 @@
 TPS/MBPS</t>
   </si>
   <si>
+    <t>Sessions</t>
+  </si>
+  <si>
     <t>Firewall + AppSec(Unified policy)</t>
   </si>
   <si>
-    <t>6930 TPS / 3995 Mbps</t>
+    <t>10600 TPS / 3995 Mbps</t>
   </si>
   <si>
     <t>*100 Sessions</t>
@@ -1162,6 +1166,9 @@
     <t>** Has to be re-tested with more ports</t>
   </si>
   <si>
+    <t>1920 CPS/ 1025 Mbos</t>
+  </si>
+  <si>
     <t>1085 CPS / 622 Mbps</t>
   </si>
   <si>
@@ -1228,12 +1235,12 @@
     <t>135 CPS / 81 Mbps</t>
   </si>
   <si>
+    <t>800 TPS / 315 Mbps</t>
+  </si>
+  <si>
     <t>CPS</t>
   </si>
   <si>
-    <t>Sessions</t>
-  </si>
-  <si>
     <t>744.1 KPPS/500 Mbps</t>
   </si>
   <si>
@@ -1283,6 +1290,96 @@
   </si>
   <si>
     <t>Max UTM- NG-WF Sessions capacity</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="18"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Release: 25.4X300-D10-202605310154.0-EVO
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Testcase Description</t>
+  </si>
+  <si>
+    <t>Global data shm / Comments</t>
+  </si>
+  <si>
+    <t>AppSec - HTTP Throughput (64KB)</t>
+  </si>
+  <si>
+    <t>1650 CPS / 920 Mbps</t>
+  </si>
+  <si>
+    <t>2000 CPS / 1350 Mbps</t>
+  </si>
+  <si>
+    <t>AppSec - HTTP  CPS (64B)</t>
+  </si>
+  <si>
+    <t>2400 CPS</t>
+  </si>
+  <si>
+    <t>3000 CPS</t>
+  </si>
+  <si>
+    <t>AppSec + SSL(TLS1.2) - HTTPS Throughput (64KB)</t>
+  </si>
+  <si>
+    <t>240 CPS / 140 Mbps</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <u/>
+        <sz val="18"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Release: 25.4X300-202605180407.0-EVO
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="18"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>1650 CPS/928 Mbps</t>
+  </si>
+  <si>
+    <t>240 CPS / 139 Mbps</t>
   </si>
   <si>
     <r>
@@ -1494,7 +1591,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1615,6 +1712,52 @@
     <font>
       <sz val="16"/>
       <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1884,7 +2027,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2107,10 +2250,75 @@
     <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4670,10 +4878,10 @@
       <c r="A1" s="50" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="80" t="s">
+      <c r="B1" s="101" t="s">
         <v>193</v>
       </c>
-      <c r="C1" s="81"/>
+      <c r="C1" s="102"/>
       <c r="D1" s="36" t="s">
         <v>194</v>
       </c>
@@ -5075,21 +5283,21 @@
         <v>197</v>
       </c>
       <c r="D29" s="40" t="s">
-        <v>198</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="15.95">
       <c r="A30" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C30" s="47">
         <v>77</v>
       </c>
       <c r="D30" s="24" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E30" t="s">
         <v>203</v>
@@ -5097,16 +5305,16 @@
     </row>
     <row r="31" spans="1:5" ht="15.95">
       <c r="A31" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C31" s="47">
         <v>77</v>
       </c>
       <c r="D31" s="24" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E31" t="s">
         <v>203</v>
@@ -5114,16 +5322,16 @@
     </row>
     <row r="32" spans="1:5" ht="15.95">
       <c r="A32" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C32" s="47">
         <v>77</v>
       </c>
       <c r="D32" s="24" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E32" t="s">
         <v>203</v>
@@ -5134,18 +5342,18 @@
         <v>233</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C33" s="47">
         <v>93</v>
       </c>
       <c r="D33" s="24" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="41.25" customHeight="1">
       <c r="A34" s="29" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B34" s="39" t="s">
         <v>196</v>
@@ -5159,7 +5367,7 @@
     </row>
     <row r="35" spans="1:5" ht="15.95">
       <c r="A35" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B35" s="4">
         <v>20000</v>
@@ -5173,7 +5381,7 @@
     </row>
     <row r="36" spans="1:5" ht="15.95">
       <c r="A36" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B36" s="4">
         <v>19330</v>
@@ -5187,7 +5395,7 @@
     </row>
     <row r="37" spans="1:5" ht="15.6" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B37" s="4">
         <v>10000</v>
@@ -5201,7 +5409,7 @@
     </row>
     <row r="38" spans="1:5" ht="15.95">
       <c r="A38" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B38" s="4">
         <v>2400</v>
@@ -5215,7 +5423,7 @@
     </row>
     <row r="39" spans="1:5" ht="15.95">
       <c r="A39" s="22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B39" s="15">
         <v>2250</v>
@@ -5229,7 +5437,7 @@
     </row>
     <row r="40" spans="1:5" ht="15.95">
       <c r="A40" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B40" s="45">
         <v>975</v>
@@ -5243,7 +5451,7 @@
     </row>
     <row r="41" spans="1:5" ht="15.95">
       <c r="A41" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B41" s="4">
         <v>1550</v>
@@ -5257,7 +5465,7 @@
     </row>
     <row r="42" spans="1:5" ht="15.95">
       <c r="A42" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B42" s="4">
         <v>400</v>
@@ -5271,7 +5479,7 @@
     </row>
     <row r="43" spans="1:5" ht="15.95">
       <c r="A43" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B43" s="4">
         <v>175</v>
@@ -5285,7 +5493,7 @@
     </row>
     <row r="44" spans="1:5" ht="32.25" customHeight="1">
       <c r="A44" s="29" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B44" s="39" t="s">
         <v>196</v>
@@ -5294,49 +5502,49 @@
         <v>197</v>
       </c>
       <c r="D44" s="40" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="18.600000000000001" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C45" s="33">
         <v>98</v>
       </c>
       <c r="D45" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="17.45" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C46" s="49">
         <v>98</v>
       </c>
       <c r="D46" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="15.95">
       <c r="A47" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C47" s="23">
         <v>90</v>
       </c>
       <c r="D47" s="57" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E47" t="s">
         <v>203</v>
@@ -5344,21 +5552,21 @@
     </row>
     <row r="48" spans="1:5" ht="15.95">
       <c r="A48" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C48" s="23">
         <v>98</v>
       </c>
       <c r="D48" s="59" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.95">
       <c r="A49" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B49" s="4"/>
       <c r="C49" s="23"/>
@@ -5366,38 +5574,38 @@
     </row>
     <row r="50" spans="1:4" ht="15.95">
       <c r="A50" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C50" s="23">
         <v>99</v>
       </c>
       <c r="D50" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A51" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C51" s="32">
         <v>98</v>
       </c>
       <c r="D51" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15.6" customHeight="1">
       <c r="A52" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="C52" s="23">
         <v>99</v>
@@ -5406,147 +5614,147 @@
     </row>
     <row r="53" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A53" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C53" s="31">
         <v>99</v>
       </c>
       <c r="D53" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.95">
       <c r="A54" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C54" s="23">
         <v>98</v>
       </c>
       <c r="D54" s="59" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15.95">
       <c r="A55" s="19" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C55" s="23">
         <v>98</v>
       </c>
       <c r="D55" s="59" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="17.100000000000001" customHeight="1">
       <c r="A56" s="19" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C56" s="23">
         <v>99</v>
       </c>
       <c r="D56" s="59" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15.95">
       <c r="A57" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C57" s="23">
         <v>98</v>
       </c>
       <c r="D57" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" s="58"/>
       <c r="D58" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="30" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B59" s="4"/>
       <c r="C59" s="23"/>
       <c r="D59" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="19.5" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" s="23"/>
       <c r="D60" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="18.75" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B61" s="4"/>
       <c r="C61" s="23"/>
       <c r="D61" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="17.45" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="32"/>
       <c r="D62" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="18" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="23"/>
       <c r="D63" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="18" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="53"/>
       <c r="D64" s="70" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="32.25" customHeight="1">
       <c r="A65" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B65" s="6"/>
       <c r="C65" s="52"/>
@@ -5554,10 +5762,10 @@
     </row>
     <row r="66" spans="1:4" ht="18" customHeight="1">
       <c r="A66" s="28" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B66" s="20" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C66" s="30" t="s">
         <v>197</v>
@@ -5566,7 +5774,7 @@
     </row>
     <row r="67" spans="1:4" ht="15.95">
       <c r="A67" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B67" s="24"/>
       <c r="C67" s="10"/>
@@ -5574,7 +5782,7 @@
     </row>
     <row r="68" spans="1:4" ht="15.95">
       <c r="A68" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B68" s="24"/>
       <c r="C68" s="10"/>
@@ -5582,7 +5790,7 @@
     </row>
     <row r="69" spans="1:4" ht="15.95">
       <c r="A69" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B69" s="24"/>
       <c r="C69" s="10"/>
@@ -5590,7 +5798,7 @@
     </row>
     <row r="70" spans="1:4" ht="15.95">
       <c r="A70" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B70" s="24"/>
       <c r="C70" s="10"/>
@@ -5598,7 +5806,7 @@
     </row>
     <row r="71" spans="1:4" ht="15.95">
       <c r="A71" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B71" s="24"/>
       <c r="C71" s="10"/>
@@ -5606,7 +5814,7 @@
     </row>
     <row r="72" spans="1:4" ht="15.95">
       <c r="A72" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B72" s="24"/>
       <c r="C72" s="10"/>
@@ -5614,7 +5822,7 @@
     </row>
     <row r="73" spans="1:4" ht="15.95">
       <c r="A73" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B73" s="24"/>
       <c r="C73" s="10"/>
@@ -5622,7 +5830,7 @@
     </row>
     <row r="74" spans="1:4" ht="15.95">
       <c r="A74" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B74" s="24"/>
       <c r="C74" s="10"/>
@@ -5630,7 +5838,7 @@
     </row>
     <row r="75" spans="1:4" ht="15.95">
       <c r="A75" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B75" s="24"/>
       <c r="C75" s="10"/>
@@ -5638,7 +5846,7 @@
     </row>
     <row r="76" spans="1:4" ht="15.95">
       <c r="A76" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B76" s="24"/>
       <c r="C76" s="10"/>
@@ -5646,7 +5854,7 @@
     </row>
     <row r="77" spans="1:4" ht="15.95">
       <c r="A77" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B77" s="24"/>
       <c r="C77" s="10"/>
@@ -5654,7 +5862,7 @@
     </row>
     <row r="78" spans="1:4" ht="15.95">
       <c r="A78" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B78" s="24"/>
       <c r="C78" s="10"/>
@@ -5662,7 +5870,7 @@
     </row>
     <row r="79" spans="1:4" ht="15.95">
       <c r="A79" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B79" s="24"/>
       <c r="C79" s="10"/>
@@ -5670,7 +5878,7 @@
     </row>
     <row r="80" spans="1:4" ht="15.95">
       <c r="A80" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B80" s="33"/>
       <c r="C80" s="23"/>
@@ -5678,7 +5886,7 @@
     </row>
     <row r="81" spans="1:4" ht="15.95">
       <c r="A81" s="43" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B81" s="24"/>
       <c r="C81" s="32"/>
@@ -5686,7 +5894,7 @@
     </row>
     <row r="82" spans="1:4" ht="15.95">
       <c r="A82" s="51" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B82" s="24"/>
       <c r="C82" s="32"/>
@@ -5694,7 +5902,7 @@
     </row>
     <row r="83" spans="1:4" ht="15.95">
       <c r="A83" s="22" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B83" s="33"/>
       <c r="C83" s="23"/>
@@ -5702,7 +5910,7 @@
     </row>
     <row r="84" spans="1:4" ht="15.95">
       <c r="A84" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B84" s="24"/>
       <c r="C84" s="10"/>
@@ -5710,7 +5918,7 @@
     </row>
     <row r="85" spans="1:4" ht="15.95">
       <c r="A85" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B85" s="24"/>
       <c r="C85" s="10"/>
@@ -5718,10 +5926,10 @@
     </row>
     <row r="86" spans="1:4" ht="15.95">
       <c r="A86" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C86" s="10">
         <v>10</v>
@@ -5732,10 +5940,10 @@
     </row>
     <row r="87" spans="1:4" ht="15.95">
       <c r="A87" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C87" s="10">
         <v>10</v>
@@ -5746,7 +5954,7 @@
     </row>
     <row r="88" spans="1:4" ht="15.95">
       <c r="A88" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B88" s="24"/>
       <c r="C88" s="10"/>
@@ -5754,7 +5962,7 @@
     </row>
     <row r="89" spans="1:4" ht="15.95">
       <c r="A89" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B89" s="24"/>
       <c r="C89" s="10"/>
@@ -5762,7 +5970,7 @@
     </row>
     <row r="90" spans="1:4" ht="15.95">
       <c r="A90" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B90" s="24"/>
       <c r="C90" s="10"/>
@@ -5770,7 +5978,7 @@
     </row>
     <row r="91" spans="1:4" ht="15.95">
       <c r="A91" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B91" s="10">
         <v>80000</v>
@@ -5784,7 +5992,7 @@
     </row>
     <row r="92" spans="1:4" ht="15.95">
       <c r="A92" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B92" s="24">
         <v>80000</v>
@@ -5798,19 +6006,19 @@
     </row>
     <row r="93" spans="1:4" ht="15.95">
       <c r="A93" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B93" s="70">
         <v>51000</v>
       </c>
       <c r="C93" s="57"/>
       <c r="D93" s="71" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.95">
       <c r="A94" s="2" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B94" s="24">
         <v>32000</v>
@@ -5824,7 +6032,7 @@
     </row>
     <row r="95" spans="1:4" ht="15.95">
       <c r="A95" s="2" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B95" s="24">
         <v>32000</v>
@@ -5838,7 +6046,7 @@
     </row>
     <row r="96" spans="1:4" ht="15.95">
       <c r="A96" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B96" s="34">
         <v>8000</v>
@@ -5852,19 +6060,19 @@
     </row>
     <row r="97" spans="1:9" ht="15.95">
       <c r="A97" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B97" s="72">
         <v>26000</v>
       </c>
       <c r="C97" s="70"/>
       <c r="D97" s="70" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="15.95">
       <c r="A98" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B98" s="24">
         <v>1000</v>
@@ -5878,7 +6086,7 @@
     </row>
     <row r="99" spans="1:9" ht="15.95">
       <c r="A99" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B99" s="24">
         <v>300</v>
@@ -5892,7 +6100,7 @@
     </row>
     <row r="100" spans="1:9" ht="15.95">
       <c r="A100" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B100" s="16"/>
       <c r="C100" s="10"/>
@@ -5900,7 +6108,7 @@
     </row>
     <row r="101" spans="1:9" ht="15.95">
       <c r="A101" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B101" s="10"/>
       <c r="C101" s="10"/>
@@ -5908,7 +6116,7 @@
     </row>
     <row r="102" spans="1:9" ht="15.95">
       <c r="A102" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B102" s="24"/>
       <c r="C102" s="10"/>
@@ -5953,15 +6161,15 @@
   <sheetData>
     <row r="1" spans="1:5" ht="57" customHeight="1">
       <c r="A1" s="50" t="s">
-        <v>351</v>
-      </c>
-      <c r="B1" s="37" t="s">
         <v>352</v>
       </c>
-      <c r="C1" s="36" t="s">
+      <c r="B1" s="101" t="s">
+        <v>353</v>
+      </c>
+      <c r="C1" s="102"/>
+      <c r="D1" s="36" t="s">
         <v>194</v>
       </c>
-      <c r="D1" s="17"/>
     </row>
     <row r="2" spans="1:5" ht="18" customHeight="1">
       <c r="A2" s="38" t="s">
@@ -5982,7 +6190,7 @@
         <v>199</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="C3" s="59">
         <v>91</v>
@@ -5996,7 +6204,7 @@
         <v>201</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C4" s="4">
         <v>70</v>
@@ -6005,23 +6213,29 @@
         <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.6" customHeight="1">
       <c r="A5" s="2" t="s">
         <v>204</v>
       </c>
-      <c r="B5" s="4"/>
-      <c r="C5" s="4"/>
-      <c r="D5" s="59"/>
+      <c r="B5" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="C5" s="4">
+        <v>92</v>
+      </c>
+      <c r="D5" s="59">
+        <v>57</v>
+      </c>
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1">
       <c r="A6" s="2" t="s">
         <v>206</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C6" s="4">
         <v>94</v>
@@ -6035,7 +6249,7 @@
         <v>208</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C7" s="59">
         <v>96</v>
@@ -6049,7 +6263,7 @@
         <v>210</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C8" s="4">
         <v>90</v>
@@ -6063,7 +6277,7 @@
         <v>212</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="C9" s="59">
         <v>90</v>
@@ -6077,7 +6291,7 @@
         <v>214</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C10" s="4">
         <v>90</v>
@@ -6086,12 +6300,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" ht="15.95">
       <c r="A11" s="2" t="s">
         <v>216</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="C11" s="4">
         <v>92</v>
@@ -6100,7 +6314,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" ht="15.95">
       <c r="A12" s="2" t="s">
         <v>218</v>
       </c>
@@ -6119,7 +6333,7 @@
         <v>220</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C13" s="4">
         <v>90</v>
@@ -6133,7 +6347,7 @@
         <v>222</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C14" s="4">
         <v>90</v>
@@ -6147,7 +6361,7 @@
         <v>224</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C15" s="4">
         <v>94</v>
@@ -6156,12 +6370,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" ht="15.95">
       <c r="A16" s="3" t="s">
         <v>226</v>
       </c>
       <c r="B16" s="46" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C16" s="4">
         <v>92</v>
@@ -6170,12 +6384,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" ht="15.95">
       <c r="A17" s="43" t="s">
         <v>228</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="C17" s="7">
         <v>92</v>
@@ -6189,7 +6403,7 @@
         <v>230</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>197</v>
@@ -6203,7 +6417,7 @@
         <v>231</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C19" s="55">
         <v>92</v>
@@ -6217,7 +6431,7 @@
         <v>233</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C20" s="57">
         <v>95</v>
@@ -6231,7 +6445,7 @@
         <v>235</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="C21" s="57">
         <v>95</v>
@@ -6245,7 +6459,7 @@
         <v>237</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C22" s="57">
         <v>93</v>
@@ -6259,7 +6473,7 @@
         <v>239</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C23" s="57">
         <v>92</v>
@@ -6273,7 +6487,7 @@
         <v>241</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C24" s="57">
         <v>92</v>
@@ -6282,7 +6496,7 @@
         <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.95">
@@ -6290,7 +6504,7 @@
         <v>243</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="C25" s="57">
         <v>92</v>
@@ -6304,7 +6518,7 @@
         <v>245</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="C26" s="57">
         <v>90</v>
@@ -6318,7 +6532,7 @@
         <v>247</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C27" s="57">
         <v>90</v>
@@ -6332,7 +6546,7 @@
         <v>249</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="C28" s="57">
         <v>92</v>
@@ -6346,53 +6560,86 @@
         <v>251</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>197</v>
       </c>
       <c r="D29" s="40" t="s">
-        <v>198</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="15.95">
       <c r="A30" s="2" t="s">
-        <v>253</v>
-      </c>
-      <c r="B30" s="47"/>
-      <c r="C30" s="57"/>
-      <c r="D30" s="59"/>
+        <v>254</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C30" s="47">
+        <v>68</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="E30" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="31" spans="1:6" ht="15.95">
       <c r="A31" s="2" t="s">
+        <v>257</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C31" s="47">
+        <v>68</v>
+      </c>
+      <c r="D31" s="24" t="s">
         <v>256</v>
       </c>
-      <c r="B31" s="47"/>
-      <c r="C31" s="57"/>
-      <c r="D31" s="59"/>
+      <c r="E31" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="32" spans="1:6" ht="15.95">
       <c r="A32" s="2" t="s">
-        <v>257</v>
-      </c>
-      <c r="B32" s="47"/>
-      <c r="C32" s="57"/>
-      <c r="D32" s="59"/>
+        <v>258</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C32" s="47">
+        <v>68</v>
+      </c>
+      <c r="D32" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="E32" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="33" spans="1:4" ht="17.45" customHeight="1">
       <c r="A33" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="B33" s="47"/>
-      <c r="C33" s="54"/>
-      <c r="D33" s="59"/>
+      <c r="B33" s="47" t="s">
+        <v>380</v>
+      </c>
+      <c r="C33" s="57">
+        <v>92</v>
+      </c>
+      <c r="D33" s="24" t="s">
+        <v>256</v>
+      </c>
     </row>
     <row r="34" spans="1:4" ht="18" customHeight="1">
       <c r="A34" s="29" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="C34" s="40" t="s">
         <v>197</v>
@@ -6403,7 +6650,7 @@
     </row>
     <row r="35" spans="1:4" ht="15.95">
       <c r="A35" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B35" s="48">
         <v>26000</v>
@@ -6417,7 +6664,7 @@
     </row>
     <row r="36" spans="1:4" ht="15.95">
       <c r="A36" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B36" s="4">
         <v>25400</v>
@@ -6431,7 +6678,7 @@
     </row>
     <row r="37" spans="1:4" ht="15.6" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B37" s="4">
         <v>13300</v>
@@ -6445,7 +6692,7 @@
     </row>
     <row r="38" spans="1:4" ht="15.95">
       <c r="A38" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B38" s="4">
         <v>3200</v>
@@ -6459,7 +6706,7 @@
     </row>
     <row r="39" spans="1:4" ht="15.95">
       <c r="A39" s="22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B39" s="15">
         <v>2700</v>
@@ -6471,9 +6718,9 @@
         <v>69</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
+    <row r="40" spans="1:4" ht="15.95">
       <c r="A40" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B40" s="45">
         <v>1050</v>
@@ -6487,7 +6734,7 @@
     </row>
     <row r="41" spans="1:4" ht="15.95">
       <c r="A41" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B41" s="4">
         <v>1810</v>
@@ -6501,7 +6748,7 @@
     </row>
     <row r="42" spans="1:4" ht="15.95">
       <c r="A42" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B42" s="1">
         <v>460</v>
@@ -6515,7 +6762,7 @@
     </row>
     <row r="43" spans="1:4" ht="15.95">
       <c r="A43" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B43" s="4">
         <v>205</v>
@@ -6529,77 +6776,77 @@
     </row>
     <row r="44" spans="1:4" ht="18" customHeight="1">
       <c r="A44" s="29" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C44" s="40" t="s">
         <v>197</v>
       </c>
       <c r="D44" s="40" t="s">
-        <v>379</v>
+        <v>253</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="18.600000000000001" customHeight="1">
       <c r="A45" s="13" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C45" s="24">
         <v>98</v>
       </c>
       <c r="D45" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="17.45" customHeight="1">
       <c r="A46" s="13" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B46" s="49" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="C46" s="24">
         <v>98</v>
       </c>
       <c r="D46" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.95">
       <c r="A47" s="8" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C47" s="57">
         <v>96</v>
       </c>
       <c r="D47" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.95">
       <c r="A48" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B48" s="49" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C48" s="57">
         <v>96</v>
       </c>
       <c r="D48" s="59" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
     </row>
     <row r="49" spans="1:4" ht="15.95">
       <c r="A49" s="2" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B49" s="23"/>
       <c r="C49" s="57"/>
@@ -6607,119 +6854,119 @@
     </row>
     <row r="50" spans="1:4" ht="15.95">
       <c r="A50" s="8" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="C50" s="55">
         <v>98</v>
       </c>
       <c r="D50" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="51" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A51" s="8" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B51" s="32" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C51" s="57">
         <v>98</v>
       </c>
       <c r="D51" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="52" spans="1:4" ht="15.6" customHeight="1">
       <c r="A52" s="8" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="C52" s="57">
         <v>99</v>
       </c>
       <c r="D52" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="53" spans="1:4" ht="16.350000000000001" customHeight="1">
       <c r="A53" s="8" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B53" s="31" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C53" s="65">
         <v>99</v>
       </c>
       <c r="D53" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="54" spans="1:4" ht="15.95">
       <c r="A54" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B54" s="23" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="C54" s="66">
         <v>98</v>
       </c>
       <c r="D54" s="59" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="55" spans="1:4" ht="15.95">
       <c r="A55" s="19" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B55" s="23" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C55" s="66">
         <v>98</v>
       </c>
       <c r="D55" s="59" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="17.100000000000001" customHeight="1">
       <c r="A56" s="19" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C56" s="66">
         <v>96</v>
       </c>
       <c r="D56" s="59" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="15.95">
       <c r="A57" s="9" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B57" s="25" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="C57" s="57">
         <v>96</v>
       </c>
       <c r="D57" s="59" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="17.25" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B58" s="23"/>
       <c r="C58" s="55"/>
@@ -6727,7 +6974,7 @@
     </row>
     <row r="59" spans="1:4" ht="30" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B59" s="23"/>
       <c r="C59" s="57"/>
@@ -6735,7 +6982,7 @@
     </row>
     <row r="60" spans="1:4" ht="19.5" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B60" s="23"/>
       <c r="C60" s="57"/>
@@ -6743,7 +6990,7 @@
     </row>
     <row r="61" spans="1:4" ht="18.75" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B61" s="23"/>
       <c r="C61" s="57"/>
@@ -6751,7 +6998,7 @@
     </row>
     <row r="62" spans="1:4" ht="17.45" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B62" s="32"/>
       <c r="C62" s="57"/>
@@ -6759,7 +7006,7 @@
     </row>
     <row r="63" spans="1:4" ht="18" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B63" s="23"/>
       <c r="C63" s="57"/>
@@ -6767,7 +7014,7 @@
     </row>
     <row r="64" spans="1:4" ht="18" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B64" s="53"/>
       <c r="C64" s="57"/>
@@ -6775,7 +7022,7 @@
     </row>
     <row r="65" spans="1:4" ht="32.25" customHeight="1">
       <c r="A65" s="3" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B65" s="52"/>
       <c r="C65" s="57"/>
@@ -6783,21 +7030,21 @@
     </row>
     <row r="66" spans="1:4" ht="18" customHeight="1">
       <c r="A66" s="28" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B66" s="30" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="C66" s="67" t="s">
         <v>197</v>
       </c>
       <c r="D66" s="67" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="15.95">
       <c r="A67" s="2" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B67" s="10"/>
       <c r="C67" s="57"/>
@@ -6805,7 +7052,7 @@
     </row>
     <row r="68" spans="1:4" ht="15.95">
       <c r="A68" s="2" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B68" s="10"/>
       <c r="C68" s="57"/>
@@ -6813,7 +7060,7 @@
     </row>
     <row r="69" spans="1:4" ht="15.95">
       <c r="A69" s="2" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B69" s="10"/>
       <c r="C69" s="57"/>
@@ -6821,7 +7068,7 @@
     </row>
     <row r="70" spans="1:4" ht="15.95">
       <c r="A70" s="2" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B70" s="10"/>
       <c r="C70" s="57"/>
@@ -6829,7 +7076,7 @@
     </row>
     <row r="71" spans="1:4" ht="15.95">
       <c r="A71" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B71" s="10"/>
       <c r="C71" s="57"/>
@@ -6837,7 +7084,7 @@
     </row>
     <row r="72" spans="1:4" ht="15.95">
       <c r="A72" s="2" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B72" s="10"/>
       <c r="C72" s="57"/>
@@ -6845,7 +7092,7 @@
     </row>
     <row r="73" spans="1:4" ht="15.95">
       <c r="A73" s="2" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B73" s="10"/>
       <c r="C73" s="57"/>
@@ -6853,7 +7100,7 @@
     </row>
     <row r="74" spans="1:4" ht="15.95">
       <c r="A74" s="2" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B74" s="10">
         <v>1536</v>
@@ -6863,7 +7110,7 @@
     </row>
     <row r="75" spans="1:4" ht="15.95">
       <c r="A75" s="2" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B75" s="10"/>
       <c r="C75" s="57"/>
@@ -6871,7 +7118,7 @@
     </row>
     <row r="76" spans="1:4" ht="15.95">
       <c r="A76" s="2" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B76" s="10"/>
       <c r="C76" s="57"/>
@@ -6879,7 +7126,7 @@
     </row>
     <row r="77" spans="1:4" ht="15.95">
       <c r="A77" s="2" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B77" s="10"/>
       <c r="C77" s="57"/>
@@ -6887,7 +7134,7 @@
     </row>
     <row r="78" spans="1:4" ht="15.95">
       <c r="A78" s="2" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B78" s="10"/>
       <c r="C78" s="57"/>
@@ -6895,7 +7142,7 @@
     </row>
     <row r="79" spans="1:4" ht="15.95">
       <c r="A79" s="2" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B79" s="10"/>
       <c r="C79" s="57"/>
@@ -6903,7 +7150,7 @@
     </row>
     <row r="80" spans="1:4" ht="15.95">
       <c r="A80" s="2" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B80" s="23"/>
       <c r="C80" s="57"/>
@@ -6911,7 +7158,7 @@
     </row>
     <row r="81" spans="1:4" ht="15.95">
       <c r="A81" s="43" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B81" s="32"/>
       <c r="C81" s="57"/>
@@ -6919,7 +7166,7 @@
     </row>
     <row r="82" spans="1:4" ht="15.95">
       <c r="A82" s="51" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B82" s="32"/>
       <c r="C82" s="57"/>
@@ -6927,7 +7174,7 @@
     </row>
     <row r="83" spans="1:4" ht="15.95">
       <c r="A83" s="22" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B83" s="23"/>
       <c r="C83" s="57"/>
@@ -6935,7 +7182,7 @@
     </row>
     <row r="84" spans="1:4" ht="15.95">
       <c r="A84" s="2" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B84" s="10"/>
       <c r="C84" s="57"/>
@@ -6943,7 +7190,7 @@
     </row>
     <row r="85" spans="1:4" ht="15.95">
       <c r="A85" s="2" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B85" s="10"/>
       <c r="C85" s="57"/>
@@ -6951,10 +7198,10 @@
     </row>
     <row r="86" spans="1:4" ht="15.95">
       <c r="A86" s="2" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C86" s="10">
         <v>10</v>
@@ -6965,10 +7212,10 @@
     </row>
     <row r="87" spans="1:4" ht="15.95">
       <c r="A87" s="2" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B87" s="10" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C87" s="10">
         <v>10</v>
@@ -6979,7 +7226,7 @@
     </row>
     <row r="88" spans="1:4" ht="15.95">
       <c r="A88" s="2" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B88" s="10"/>
       <c r="C88" s="57"/>
@@ -6987,7 +7234,7 @@
     </row>
     <row r="89" spans="1:4" ht="15.95">
       <c r="A89" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B89" s="10"/>
       <c r="C89" s="57"/>
@@ -6995,7 +7242,7 @@
     </row>
     <row r="90" spans="1:4" ht="15.95">
       <c r="A90" s="2" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B90" s="10"/>
       <c r="C90" s="57"/>
@@ -7003,7 +7250,7 @@
     </row>
     <row r="91" spans="1:4" ht="15.95">
       <c r="A91" s="2" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B91" s="10">
         <v>96000</v>
@@ -7017,7 +7264,7 @@
     </row>
     <row r="92" spans="1:4" ht="15.95">
       <c r="A92" s="2" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B92" s="10">
         <v>96000</v>
@@ -7031,19 +7278,19 @@
     </row>
     <row r="93" spans="1:4" ht="15.95">
       <c r="A93" s="2" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B93" s="70">
         <v>51000</v>
       </c>
       <c r="C93" s="57"/>
       <c r="D93" s="71" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.95">
       <c r="A94" s="2" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B94" s="73"/>
       <c r="C94" s="56"/>
@@ -7051,7 +7298,7 @@
     </row>
     <row r="95" spans="1:4" ht="15.95">
       <c r="A95" s="2" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B95" s="26"/>
       <c r="C95" s="56"/>
@@ -7059,7 +7306,7 @@
     </row>
     <row r="96" spans="1:4" ht="15.95">
       <c r="A96" s="8" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B96" s="35"/>
       <c r="C96" s="10"/>
@@ -7067,7 +7314,7 @@
     </row>
     <row r="97" spans="1:9" ht="15.95">
       <c r="A97" s="2" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B97" s="10"/>
       <c r="C97" s="10"/>
@@ -7075,7 +7322,7 @@
     </row>
     <row r="98" spans="1:9" ht="15.95">
       <c r="A98" s="2" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B98" s="10">
         <v>1200</v>
@@ -7089,7 +7336,7 @@
     </row>
     <row r="99" spans="1:9" ht="15.95">
       <c r="A99" s="2" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B99" s="10"/>
       <c r="C99" s="10"/>
@@ -7097,7 +7344,7 @@
     </row>
     <row r="100" spans="1:9" ht="15.95">
       <c r="A100" s="2" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B100" s="10"/>
       <c r="C100" s="10"/>
@@ -7105,7 +7352,7 @@
     </row>
     <row r="101" spans="1:9" ht="15.95">
       <c r="A101" s="2" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="B101" s="10"/>
       <c r="C101" s="10"/>
@@ -7113,7 +7360,7 @@
     </row>
     <row r="102" spans="1:9" ht="15.95">
       <c r="A102" s="2" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B102" s="10"/>
       <c r="C102" s="10"/>
@@ -7137,11 +7384,430 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F102" xr:uid="{63A7BD36-8D88-3742-A4AC-48B0AFB67141}"/>
+  <mergeCells count="1">
+    <mergeCell ref="B1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F1F4FD9-0BA8-D443-A42F-4E5E606C52A0}">
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr defaultColWidth="62.42578125" defaultRowHeight="24"/>
+  <cols>
+    <col min="1" max="1" width="134.85546875" style="82" customWidth="1"/>
+    <col min="2" max="2" width="31.140625" style="82" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.140625" style="82" customWidth="1"/>
+    <col min="4" max="4" width="26" style="82" customWidth="1"/>
+    <col min="5" max="5" width="47.7109375" style="82" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" style="82" customWidth="1"/>
+    <col min="7" max="7" width="33.85546875" style="82" customWidth="1"/>
+    <col min="8" max="16384" width="62.42578125" style="82"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="75">
+      <c r="A1" s="80" t="s">
+        <v>399</v>
+      </c>
+      <c r="B1" s="103" t="s">
+        <v>193</v>
+      </c>
+      <c r="C1" s="104"/>
+      <c r="D1" s="81" t="s">
+        <v>194</v>
+      </c>
+      <c r="E1" s="103" t="s">
+        <v>353</v>
+      </c>
+      <c r="F1" s="104"/>
+      <c r="G1" s="81" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="50.1">
+      <c r="A2" s="83" t="s">
+        <v>400</v>
+      </c>
+      <c r="B2" s="84" t="s">
+        <v>369</v>
+      </c>
+      <c r="C2" s="85" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="84" t="s">
+        <v>401</v>
+      </c>
+      <c r="E2" s="84" t="s">
+        <v>196</v>
+      </c>
+      <c r="F2" s="85" t="s">
+        <v>197</v>
+      </c>
+      <c r="G2" s="85" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="24.95">
+      <c r="A3" s="86" t="s">
+        <v>402</v>
+      </c>
+      <c r="B3" s="87" t="s">
+        <v>403</v>
+      </c>
+      <c r="C3" s="88">
+        <v>94</v>
+      </c>
+      <c r="D3" s="89">
+        <v>40</v>
+      </c>
+      <c r="E3" s="87" t="s">
+        <v>404</v>
+      </c>
+      <c r="F3" s="88">
+        <v>93</v>
+      </c>
+      <c r="G3" s="89">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="24.95">
+      <c r="A4" s="86" t="s">
+        <v>405</v>
+      </c>
+      <c r="B4" s="89" t="s">
+        <v>406</v>
+      </c>
+      <c r="C4" s="90">
+        <v>95</v>
+      </c>
+      <c r="D4" s="91">
+        <v>40</v>
+      </c>
+      <c r="E4" s="89" t="s">
+        <v>407</v>
+      </c>
+      <c r="F4" s="90">
+        <v>94</v>
+      </c>
+      <c r="G4" s="91">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="24.95">
+      <c r="A5" s="86" t="s">
+        <v>408</v>
+      </c>
+      <c r="B5" s="92" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="93">
+        <v>94</v>
+      </c>
+      <c r="D5" s="94">
+        <v>60</v>
+      </c>
+      <c r="E5" s="92" t="s">
+        <v>409</v>
+      </c>
+      <c r="F5" s="93">
+        <v>91</v>
+      </c>
+      <c r="G5" s="94">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="24.95">
+      <c r="A6" s="95" t="s">
+        <v>271</v>
+      </c>
+      <c r="B6" s="89" t="s">
+        <v>272</v>
+      </c>
+      <c r="C6" s="96">
+        <v>99</v>
+      </c>
+      <c r="D6" s="97" t="s">
+        <v>273</v>
+      </c>
+      <c r="E6" s="89" t="s">
+        <v>382</v>
+      </c>
+      <c r="F6" s="89">
+        <v>98</v>
+      </c>
+      <c r="G6" s="97" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="24.95">
+      <c r="A7" s="95" t="s">
+        <v>274</v>
+      </c>
+      <c r="B7" s="89" t="s">
+        <v>275</v>
+      </c>
+      <c r="C7" s="98">
+        <v>99</v>
+      </c>
+      <c r="D7" s="97" t="s">
+        <v>273</v>
+      </c>
+      <c r="E7" s="89" t="s">
+        <v>383</v>
+      </c>
+      <c r="F7" s="89">
+        <v>98</v>
+      </c>
+      <c r="G7" s="97" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="24.95">
+      <c r="A8" s="99" t="s">
+        <v>276</v>
+      </c>
+      <c r="B8" s="92" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" s="93">
+        <v>90</v>
+      </c>
+      <c r="D8" s="94" t="s">
+        <v>273</v>
+      </c>
+      <c r="E8" s="89" t="s">
+        <v>384</v>
+      </c>
+      <c r="F8" s="89">
+        <v>96</v>
+      </c>
+      <c r="G8" s="94" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="47.25">
+      <c r="A9" s="86" t="s">
+        <v>303</v>
+      </c>
+      <c r="B9" s="89"/>
+      <c r="C9" s="93"/>
+      <c r="D9" s="100" t="s">
+        <v>302</v>
+      </c>
+      <c r="E9" s="89"/>
+      <c r="F9" s="93"/>
+      <c r="G9" s="100" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="75">
+      <c r="A12" s="80" t="s">
+        <v>410</v>
+      </c>
+      <c r="B12" s="103" t="s">
+        <v>193</v>
+      </c>
+      <c r="C12" s="104"/>
+      <c r="D12" s="81" t="s">
+        <v>194</v>
+      </c>
+      <c r="E12" s="103" t="s">
+        <v>353</v>
+      </c>
+      <c r="F12" s="104"/>
+      <c r="G12" s="81" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="50.1">
+      <c r="A13" s="83" t="s">
+        <v>400</v>
+      </c>
+      <c r="B13" s="84" t="s">
+        <v>369</v>
+      </c>
+      <c r="C13" s="85" t="s">
+        <v>197</v>
+      </c>
+      <c r="D13" s="84" t="s">
+        <v>401</v>
+      </c>
+      <c r="E13" s="84" t="s">
+        <v>196</v>
+      </c>
+      <c r="F13" s="85" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="85" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="24.95">
+      <c r="A14" s="86" t="s">
+        <v>402</v>
+      </c>
+      <c r="B14" s="87" t="s">
+        <v>411</v>
+      </c>
+      <c r="C14" s="88">
+        <v>95</v>
+      </c>
+      <c r="D14" s="89">
+        <v>61</v>
+      </c>
+      <c r="E14" s="87" t="s">
+        <v>404</v>
+      </c>
+      <c r="F14" s="88">
+        <v>93</v>
+      </c>
+      <c r="G14" s="89">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="24.95">
+      <c r="A15" s="86" t="s">
+        <v>405</v>
+      </c>
+      <c r="B15" s="89" t="s">
+        <v>406</v>
+      </c>
+      <c r="C15" s="90">
+        <v>95</v>
+      </c>
+      <c r="D15" s="91">
+        <v>61</v>
+      </c>
+      <c r="E15" s="89" t="s">
+        <v>407</v>
+      </c>
+      <c r="F15" s="90">
+        <v>94</v>
+      </c>
+      <c r="G15" s="91">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="24.95">
+      <c r="A16" s="86" t="s">
+        <v>408</v>
+      </c>
+      <c r="B16" s="92" t="s">
+        <v>234</v>
+      </c>
+      <c r="C16" s="93">
+        <v>94</v>
+      </c>
+      <c r="D16" s="94">
+        <v>60</v>
+      </c>
+      <c r="E16" s="92" t="s">
+        <v>412</v>
+      </c>
+      <c r="F16" s="93">
+        <v>91</v>
+      </c>
+      <c r="G16" s="94">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="24.95">
+      <c r="A17" s="95" t="s">
+        <v>271</v>
+      </c>
+      <c r="B17" s="89" t="s">
+        <v>272</v>
+      </c>
+      <c r="C17" s="96">
+        <v>99</v>
+      </c>
+      <c r="D17" s="97" t="s">
+        <v>273</v>
+      </c>
+      <c r="E17" s="89" t="s">
+        <v>382</v>
+      </c>
+      <c r="F17" s="89">
+        <v>98</v>
+      </c>
+      <c r="G17" s="97" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="24.95">
+      <c r="A18" s="95" t="s">
+        <v>274</v>
+      </c>
+      <c r="B18" s="89" t="s">
+        <v>275</v>
+      </c>
+      <c r="C18" s="98">
+        <v>99</v>
+      </c>
+      <c r="D18" s="97" t="s">
+        <v>273</v>
+      </c>
+      <c r="E18" s="89" t="s">
+        <v>383</v>
+      </c>
+      <c r="F18" s="89">
+        <v>98</v>
+      </c>
+      <c r="G18" s="97" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="24.95">
+      <c r="A19" s="99" t="s">
+        <v>276</v>
+      </c>
+      <c r="B19" s="92" t="s">
+        <v>277</v>
+      </c>
+      <c r="C19" s="93">
+        <v>90</v>
+      </c>
+      <c r="D19" s="94" t="s">
+        <v>273</v>
+      </c>
+      <c r="E19" s="89" t="s">
+        <v>384</v>
+      </c>
+      <c r="F19" s="89">
+        <v>96</v>
+      </c>
+      <c r="G19" s="94" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="47.25">
+      <c r="A20" s="86" t="s">
+        <v>303</v>
+      </c>
+      <c r="B20" s="89"/>
+      <c r="C20" s="93"/>
+      <c r="D20" s="100" t="s">
+        <v>302</v>
+      </c>
+      <c r="E20" s="89"/>
+      <c r="F20" s="93"/>
+      <c r="G20" s="100" t="s">
+        <v>302</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="E1:F1"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="E12:F12"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D8EE6899-576B-F44E-A189-C616F2524B03}">
   <dimension ref="A1:C46"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
@@ -7153,10 +7819,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="60">
       <c r="A1" s="50" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C1" s="36" t="s">
         <v>194</v>
@@ -7167,34 +7833,34 @@
         <v>195</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C2" s="40"/>
     </row>
     <row r="3" spans="1:3" ht="18.95" hidden="1">
       <c r="A3" s="22" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="42"/>
     </row>
     <row r="4" spans="1:3" ht="15.95" hidden="1">
       <c r="A4" s="2" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="15.95" hidden="1">
       <c r="A5" s="2" t="s">
-        <v>400</v>
+        <v>416</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="59"/>
     </row>
     <row r="6" spans="1:3" ht="15.95" hidden="1">
       <c r="A6" s="2" t="s">
-        <v>401</v>
+        <v>417</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -7211,10 +7877,10 @@
         <v>206</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="C8" s="60" t="s">
-        <v>403</v>
+        <v>419</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.95">
@@ -7222,10 +7888,10 @@
         <v>208</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>404</v>
+        <v>420</v>
       </c>
       <c r="C9" s="59" t="s">
-        <v>405</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.95" hidden="1">
@@ -7258,14 +7924,14 @@
     </row>
     <row r="14" spans="1:3" ht="15.95" hidden="1">
       <c r="A14" s="2" t="s">
-        <v>406</v>
+        <v>422</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" ht="15.95" hidden="1">
       <c r="A15" s="2" t="s">
-        <v>407</v>
+        <v>423</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -7324,10 +7990,10 @@
         <v>233</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>408</v>
+        <v>424</v>
       </c>
       <c r="C23" s="57" t="s">
-        <v>409</v>
+        <v>425</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.95" hidden="1">
@@ -7342,10 +8008,10 @@
         <v>237</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>410</v>
+        <v>426</v>
       </c>
       <c r="C25" s="57" t="s">
-        <v>411</v>
+        <v>427</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.95">
@@ -7353,10 +8019,10 @@
         <v>239</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="C26" s="57" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.95" hidden="1">
@@ -7403,21 +8069,21 @@
     </row>
     <row r="33" spans="1:3" ht="15.95" hidden="1">
       <c r="A33" s="2" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B33" s="47"/>
       <c r="C33" s="57"/>
     </row>
     <row r="34" spans="1:3" ht="15.95" hidden="1">
       <c r="A34" s="2" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B34" s="47"/>
       <c r="C34" s="57"/>
     </row>
     <row r="35" spans="1:3" ht="15.95" hidden="1">
       <c r="A35" s="2" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B35" s="47"/>
       <c r="C35" s="57"/>
@@ -7431,82 +8097,82 @@
     </row>
     <row r="37" spans="1:3" ht="18.95">
       <c r="A37" s="29" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B37" s="12"/>
       <c r="C37" s="63"/>
     </row>
     <row r="38" spans="1:3" ht="15.95" hidden="1">
       <c r="A38" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B38" s="48"/>
       <c r="C38" s="64"/>
     </row>
     <row r="39" spans="1:3" ht="15.95" hidden="1">
       <c r="A39" s="2" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B39" s="4"/>
       <c r="C39" s="64"/>
     </row>
     <row r="40" spans="1:3" ht="15.95">
       <c r="A40" s="2" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="C40" s="60" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.95">
       <c r="A41" s="2" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="C41" s="60" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.95" hidden="1">
       <c r="A42" s="22" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B42" s="15"/>
       <c r="C42" s="15"/>
     </row>
     <row r="43" spans="1:3" ht="15.95" hidden="1">
       <c r="A43" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B43" s="45"/>
       <c r="C43" s="15"/>
     </row>
     <row r="44" spans="1:3" ht="15.95" hidden="1">
       <c r="A44" s="2" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B44" s="4"/>
       <c r="C44" s="4"/>
     </row>
     <row r="45" spans="1:3" ht="15.95">
       <c r="A45" s="2" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15.95" hidden="1">
       <c r="A46" s="2" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -7516,7 +8182,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DA07167-CEB4-F64B-93AF-8A8BA2B4D0FF}">
   <dimension ref="A1:D14"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
@@ -7528,115 +8194,115 @@
   <sheetData>
     <row r="1" spans="1:4" ht="81">
       <c r="A1" s="76" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="B1" s="77" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="C1" s="78" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="21.95">
       <c r="A2" s="74" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="B2" s="75" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="C2" s="75" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95">
       <c r="A3" s="74" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="B3" s="75" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="C3" s="75" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="21.95">
       <c r="A4" s="74" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="B4" s="79" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="C4" s="79" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="21.95">
       <c r="A5" s="74" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="B5" s="79" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="C5" s="79" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="21.95">
       <c r="A6" s="74" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
       <c r="B6" s="75" t="s">
-        <v>432</v>
+        <v>448</v>
       </c>
       <c r="C6" s="75" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="21.95">
       <c r="A7" s="74" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
       <c r="B7" s="75" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
       <c r="C7" s="75" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
       <c r="D7" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="21.95">
       <c r="A8" s="74" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
       <c r="B8" s="75" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C8" s="75" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="D8" t="s">
-        <v>440</v>
+        <v>456</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="21.95">
       <c r="A9" s="74" t="s">
-        <v>441</v>
+        <v>457</v>
       </c>
       <c r="B9" s="75" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="C9" s="75" t="s">
-        <v>443</v>
+        <v>459</v>
       </c>
       <c r="D9" t="s">
-        <v>444</v>
+        <v>460</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="21.95">
       <c r="A10" s="74" t="s">
-        <v>445</v>
+        <v>461</v>
       </c>
       <c r="B10" s="75">
         <v>26000</v>
@@ -7647,7 +8313,7 @@
     </row>
     <row r="11" spans="1:4" ht="21.95">
       <c r="A11" s="74" t="s">
-        <v>446</v>
+        <v>462</v>
       </c>
       <c r="B11" s="75">
         <v>445</v>
@@ -7658,7 +8324,7 @@
     </row>
     <row r="12" spans="1:4" ht="21.95">
       <c r="A12" s="74" t="s">
-        <v>447</v>
+        <v>463</v>
       </c>
       <c r="B12" s="75">
         <v>96000</v>
@@ -7669,7 +8335,7 @@
     </row>
     <row r="13" spans="1:4" ht="21.95">
       <c r="A13" s="74" t="s">
-        <v>448</v>
+        <v>464</v>
       </c>
       <c r="B13" s="75">
         <v>400000</v>
@@ -7680,7 +8346,7 @@
     </row>
     <row r="14" spans="1:4" ht="21.95">
       <c r="A14" s="74" t="s">
-        <v>449</v>
+        <v>465</v>
       </c>
       <c r="B14" s="75">
         <v>200000</v>

</xml_diff>

<commit_message>
Update SRX4XX datasheet data
</commit_message>
<xml_diff>
--- a/public/data/SRX4XX_Datasheet.xlsx
+++ b/public/data/SRX4XX_Datasheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpe-my.sharepoint.com/personal/antony-ruban_alexis_hpe_com/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1023" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3FC1C92-17E6-495D-84E3-3D79CA451DA0}"/>
+  <xr:revisionPtr revIDLastSave="1038" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7558ED8-9BDD-4EEE-BA08-1951C09F4E01}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="36000" windowHeight="19740" firstSheet="2" activeTab="2" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19740" firstSheet="1" activeTab="2" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
   </bookViews>
   <sheets>
     <sheet name="ISSUES-PR's" sheetId="7" r:id="rId1"/>
@@ -22,7 +22,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'ISSUES-PR''s'!$A$1:$I$224</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SRX440'!$A$1:$F$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'SRX440'!$A$1:$F$100</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2270" uniqueCount="473">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2267" uniqueCount="471">
   <si>
     <t>number</t>
   </si>
@@ -948,9 +948,6 @@
     <t>Max IPSec VPN Tunnels supported</t>
   </si>
   <si>
-    <t>Juniper Secure Connect Scale</t>
-  </si>
-  <si>
     <t>Max GRE supported Tunnels</t>
   </si>
   <si>
@@ -991,9 +988,6 @@
   </si>
   <si>
     <t>MAX IDP(Rec policy) Sessions capacity</t>
-  </si>
-  <si>
-    <t>80K</t>
   </si>
   <si>
     <t>Max UTM-EWF Sessions capacity</t>
@@ -1229,13 +1223,10 @@
     <t>Max UTM- NG-WF Sessions capacity</t>
   </si>
   <si>
-    <t>8k</t>
-  </si>
-  <si>
-    <t>255 seconds</t>
-  </si>
-  <si>
-    <t>7 seconds</t>
+    <t>255 sec</t>
+  </si>
+  <si>
+    <t>7 sec</t>
   </si>
   <si>
     <r>
@@ -1305,7 +1296,6 @@
         <sz val="18"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Release: 25.4X300-202605180407.0-EVO
@@ -1317,7 +1307,6 @@
         <sz val="18"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -1375,6 +1364,9 @@
   </si>
   <si>
     <t>350 CPS</t>
+  </si>
+  <si>
+    <t>Release: 25.4X300-D10.2-EVO</t>
   </si>
   <si>
     <t>1650 CPS / 926 Mbps</t>
@@ -1634,7 +1626,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="26">
+  <fonts count="28">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1826,6 +1818,21 @@
       <color rgb="FF0563C1"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -2092,7 +2099,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2388,11 +2395,8 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -8854,7 +8858,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC397FCC-74C1-4D09-ACC0-E463BF5527EB}">
-  <dimension ref="A1:I106"/>
+  <dimension ref="A1:I105"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="87.85546875" customWidth="1"/>
@@ -9990,77 +9994,77 @@
       <c r="A81" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="B81" s="33"/>
-      <c r="C81" s="23"/>
+      <c r="B81" s="24">
+        <v>1750</v>
+      </c>
+      <c r="C81" s="32"/>
       <c r="D81" s="56"/>
     </row>
     <row r="82" spans="1:4" ht="15.95">
       <c r="A82" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B82" s="24">
-        <v>1750</v>
-      </c>
-      <c r="C82" s="32"/>
+      <c r="B82" s="33"/>
+      <c r="C82" s="23"/>
       <c r="D82" s="56"/>
     </row>
     <row r="83" spans="1:4" ht="15.95">
       <c r="A83" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B83" s="33"/>
-      <c r="C83" s="23"/>
+      <c r="B83" s="24"/>
+      <c r="C83" s="10"/>
       <c r="D83" s="56"/>
     </row>
     <row r="84" spans="1:4" ht="15.95">
       <c r="A84" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="B84" s="24"/>
-      <c r="C84" s="10"/>
-      <c r="D84" s="56"/>
+      <c r="B84" s="24">
+        <v>128</v>
+      </c>
+      <c r="C84" s="10">
+        <v>10</v>
+      </c>
+      <c r="D84" s="56">
+        <v>77</v>
+      </c>
     </row>
     <row r="85" spans="1:4" ht="15.95">
       <c r="A85" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="B85" s="24">
-        <v>128</v>
+      <c r="B85" s="10" t="s">
+        <v>297</v>
       </c>
       <c r="C85" s="10">
         <v>10</v>
       </c>
-      <c r="D85" s="56">
-        <v>77</v>
+      <c r="D85" s="51">
+        <v>85</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15.95">
       <c r="A86" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B86" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="C86" s="10">
         <v>10</v>
       </c>
-      <c r="D86" s="51">
+      <c r="D86" s="56">
         <v>85</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15.95">
       <c r="A87" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B87" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="C87" s="10">
-        <v>10</v>
-      </c>
-      <c r="D87" s="56">
-        <v>85</v>
-      </c>
+      <c r="B87" s="24"/>
+      <c r="C87" s="10"/>
+      <c r="D87" s="56"/>
     </row>
     <row r="88" spans="1:4" ht="15.95">
       <c r="A88" s="2" t="s">
@@ -10082,139 +10086,145 @@
       <c r="A90" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="B90" s="24"/>
-      <c r="C90" s="10"/>
-      <c r="D90" s="56"/>
+      <c r="B90" s="10">
+        <v>80000</v>
+      </c>
+      <c r="C90" s="10">
+        <v>55</v>
+      </c>
+      <c r="D90" s="56">
+        <v>35</v>
+      </c>
     </row>
     <row r="91" spans="1:4" ht="15.95">
       <c r="A91" s="2" t="s">
         <v>304</v>
       </c>
-      <c r="B91" s="10">
+      <c r="B91" s="24">
         <v>80000</v>
       </c>
       <c r="C91" s="10">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D91" s="56">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15.95">
       <c r="A92" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="B92" s="24">
+      <c r="B92" s="51">
         <v>80000</v>
       </c>
-      <c r="C92" s="10">
-        <v>60</v>
-      </c>
-      <c r="D92" s="56">
-        <v>37</v>
-      </c>
+      <c r="C92" s="56"/>
+      <c r="D92" s="67"/>
     </row>
     <row r="93" spans="1:4" ht="15.95">
       <c r="A93" s="2" t="s">
         <v>306</v>
       </c>
-      <c r="B93" s="51" t="s">
-        <v>307</v>
-      </c>
-      <c r="C93" s="56"/>
-      <c r="D93" s="67"/>
+      <c r="B93" s="24">
+        <v>80000</v>
+      </c>
+      <c r="C93" s="5">
+        <v>56</v>
+      </c>
+      <c r="D93" s="55">
+        <v>40</v>
+      </c>
     </row>
     <row r="94" spans="1:4" ht="15.95">
       <c r="A94" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B94" s="24">
+        <v>32000</v>
+      </c>
+      <c r="C94" s="26">
+        <v>57</v>
+      </c>
+      <c r="D94" s="55">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="15.95">
+      <c r="A95" s="8" t="s">
         <v>308</v>
       </c>
-      <c r="B94" s="24">
-        <v>80000</v>
-      </c>
-      <c r="C94" s="5">
-        <v>56</v>
-      </c>
-      <c r="D94" s="55">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="15.95">
-      <c r="A95" s="2" t="s">
+      <c r="B95" s="34">
+        <v>8000</v>
+      </c>
+      <c r="C95" s="35">
+        <v>74</v>
+      </c>
+      <c r="D95" s="10">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="15.95">
+      <c r="A96" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="B95" s="24">
-        <v>32000</v>
-      </c>
-      <c r="C95" s="26">
-        <v>57</v>
-      </c>
-      <c r="D95" s="55">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="15.95">
-      <c r="A96" s="8" t="s">
+      <c r="B96" s="68">
+        <v>26000</v>
+      </c>
+      <c r="C96" s="66"/>
+      <c r="D96" s="66" t="s">
         <v>310</v>
-      </c>
-      <c r="B96" s="34">
-        <v>8000</v>
-      </c>
-      <c r="C96" s="35">
-        <v>74</v>
-      </c>
-      <c r="D96" s="10">
-        <v>48</v>
       </c>
     </row>
     <row r="97" spans="1:9" ht="15.95">
       <c r="A97" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="B97" s="68">
-        <v>26000</v>
-      </c>
-      <c r="C97" s="66"/>
-      <c r="D97" s="66" t="s">
-        <v>312</v>
+      <c r="B97" s="24">
+        <v>1000</v>
+      </c>
+      <c r="C97" s="24">
+        <v>99</v>
+      </c>
+      <c r="D97" s="24">
+        <v>57</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="15.95">
       <c r="A98" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B98" s="24">
-        <v>1000</v>
-      </c>
-      <c r="C98" s="24">
+        <v>300</v>
+      </c>
+      <c r="C98" s="10">
         <v>99</v>
       </c>
-      <c r="D98" s="24">
-        <v>57</v>
+      <c r="D98" s="10">
+        <v>69</v>
       </c>
     </row>
     <row r="99" spans="1:9" ht="15.95">
       <c r="A99" s="2" t="s">
+        <v>313</v>
+      </c>
+      <c r="B99" s="16" t="s">
         <v>314</v>
       </c>
-      <c r="B99" s="24">
-        <v>300</v>
-      </c>
-      <c r="C99" s="10">
-        <v>99</v>
+      <c r="C99" s="10" t="s">
+        <v>315</v>
       </c>
       <c r="D99" s="10">
-        <v>69</v>
+        <v>75</v>
       </c>
     </row>
     <row r="100" spans="1:9" ht="15.95">
       <c r="A100" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="B100" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="C100" s="10" t="s">
         <v>315</v>
-      </c>
-      <c r="B100" s="16" t="s">
-        <v>316</v>
-      </c>
-      <c r="C100" s="10" t="s">
-        <v>317</v>
       </c>
       <c r="D100" s="10">
         <v>75</v>
@@ -10224,29 +10234,19 @@
       <c r="A101" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="B101" s="10" t="s">
-        <v>319</v>
+      <c r="B101" s="24">
+        <v>10</v>
       </c>
       <c r="C101" s="10" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="D101" s="10">
         <v>75</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="15.95">
-      <c r="A102" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="B102" s="24">
-        <v>10</v>
-      </c>
-      <c r="C102" s="10" t="s">
-        <v>317</v>
-      </c>
-      <c r="D102" s="10">
-        <v>75</v>
-      </c>
+    <row r="102" spans="1:9" ht="15" customHeight="1">
+      <c r="H102" s="11"/>
+      <c r="I102" s="11"/>
     </row>
     <row r="103" spans="1:9" ht="15" customHeight="1">
       <c r="H103" s="11"/>
@@ -10259,10 +10259,6 @@
     <row r="105" spans="1:9" ht="15" customHeight="1">
       <c r="H105" s="11"/>
       <c r="I105" s="11"/>
-    </row>
-    <row r="106" spans="1:9" ht="15" customHeight="1">
-      <c r="H106" s="11"/>
-      <c r="I106" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -10274,7 +10270,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63A7BD36-8D88-3742-A4AC-48B0AFB67141}">
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J104"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="85.140625" customWidth="1"/>
@@ -10287,10 +10283,10 @@
   <sheetData>
     <row r="1" spans="1:5" ht="57" customHeight="1">
       <c r="A1" s="50" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="B1" s="101" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C1" s="102"/>
       <c r="D1" s="36" t="s">
@@ -10316,7 +10312,7 @@
         <v>153</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C3" s="57">
         <v>91</v>
@@ -10330,7 +10326,7 @@
         <v>155</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C4" s="4">
         <v>70</v>
@@ -10339,7 +10335,7 @@
         <v>40</v>
       </c>
       <c r="E4" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.6" customHeight="1">
@@ -10347,7 +10343,7 @@
         <v>158</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C5" s="4">
         <v>92</v>
@@ -10361,7 +10357,7 @@
         <v>160</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C6" s="4">
         <v>94</v>
@@ -10375,7 +10371,7 @@
         <v>162</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="C7" s="57">
         <v>96</v>
@@ -10389,7 +10385,7 @@
         <v>164</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C8" s="4">
         <v>90</v>
@@ -10403,7 +10399,7 @@
         <v>166</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C9" s="57">
         <v>90</v>
@@ -10417,7 +10413,7 @@
         <v>168</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="C10" s="4">
         <v>90</v>
@@ -10431,7 +10427,7 @@
         <v>170</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="C11" s="4">
         <v>92</v>
@@ -10459,7 +10455,7 @@
         <v>174</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C13" s="4">
         <v>90</v>
@@ -10473,7 +10469,7 @@
         <v>176</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C14" s="4">
         <v>90</v>
@@ -10487,7 +10483,7 @@
         <v>178</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C15" s="4">
         <v>94</v>
@@ -10501,7 +10497,7 @@
         <v>180</v>
       </c>
       <c r="B16" s="46" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="C16" s="4">
         <v>92</v>
@@ -10515,7 +10511,7 @@
         <v>182</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C17" s="7">
         <v>92</v>
@@ -10529,7 +10525,7 @@
         <v>184</v>
       </c>
       <c r="B18" s="40" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C18" s="40" t="s">
         <v>151</v>
@@ -10543,7 +10539,7 @@
         <v>185</v>
       </c>
       <c r="B19" s="27" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C19" s="54">
         <v>92</v>
@@ -10557,7 +10553,7 @@
         <v>187</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="C20" s="56">
         <v>95</v>
@@ -10571,7 +10567,7 @@
         <v>189</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C21" s="56">
         <v>95</v>
@@ -10585,7 +10581,7 @@
         <v>191</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C22" s="56">
         <v>93</v>
@@ -10599,7 +10595,7 @@
         <v>193</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C23" s="56">
         <v>92</v>
@@ -10613,7 +10609,7 @@
         <v>195</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C24" s="56">
         <v>92</v>
@@ -10622,7 +10618,7 @@
         <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="15.95">
@@ -10630,7 +10626,7 @@
         <v>197</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C25" s="56">
         <v>92</v>
@@ -10644,7 +10640,7 @@
         <v>199</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="C26" s="56">
         <v>90</v>
@@ -10658,7 +10654,7 @@
         <v>201</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C27" s="56">
         <v>90</v>
@@ -10672,7 +10668,7 @@
         <v>203</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C28" s="56">
         <v>92</v>
@@ -10686,7 +10682,7 @@
         <v>205</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C29" s="40" t="s">
         <v>151</v>
@@ -10751,7 +10747,7 @@
         <v>187</v>
       </c>
       <c r="B33" s="47" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C33" s="56">
         <v>92</v>
@@ -10765,7 +10761,7 @@
         <v>214</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="C34" s="40" t="s">
         <v>151</v>
@@ -10779,7 +10775,7 @@
         <v>215</v>
       </c>
       <c r="B35" s="48" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C35" s="62">
         <v>90</v>
@@ -10974,7 +10970,7 @@
         <v>225</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C44" s="40" t="s">
         <v>151</v>
@@ -10988,7 +10984,7 @@
         <v>226</v>
       </c>
       <c r="B45" s="33" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="C45" s="24">
         <v>98</v>
@@ -11002,7 +10998,7 @@
         <v>229</v>
       </c>
       <c r="B46" s="49" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C46" s="24">
         <v>98</v>
@@ -11016,7 +11012,7 @@
         <v>231</v>
       </c>
       <c r="B47" s="23" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="C47" s="56">
         <v>96</v>
@@ -11030,7 +11026,7 @@
         <v>233</v>
       </c>
       <c r="B48" s="49" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="C48" s="56">
         <v>96</v>
@@ -11044,7 +11040,7 @@
         <v>236</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C49" s="23">
         <v>50</v>
@@ -11056,7 +11052,7 @@
         <v>238</v>
       </c>
       <c r="B50" s="23" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C50" s="54">
         <v>98</v>
@@ -11070,7 +11066,7 @@
         <v>240</v>
       </c>
       <c r="B51" s="32" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C51" s="56">
         <v>98</v>
@@ -11084,7 +11080,7 @@
         <v>242</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="C52" s="56">
         <v>99</v>
@@ -11098,7 +11094,7 @@
         <v>244</v>
       </c>
       <c r="B53" s="31" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C53" s="63">
         <v>99</v>
@@ -11112,7 +11108,7 @@
         <v>246</v>
       </c>
       <c r="B54" s="23" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C54" s="64">
         <v>98</v>
@@ -11126,7 +11122,7 @@
         <v>249</v>
       </c>
       <c r="B55" s="23" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="C55" s="64">
         <v>98</v>
@@ -11140,7 +11136,7 @@
         <v>252</v>
       </c>
       <c r="B56" s="23" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="C56" s="64">
         <v>96</v>
@@ -11154,7 +11150,7 @@
         <v>255</v>
       </c>
       <c r="B57" s="25" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C57" s="56">
         <v>96</v>
@@ -11168,7 +11164,7 @@
         <v>257</v>
       </c>
       <c r="B58" s="23" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="C58" s="54">
         <v>78</v>
@@ -11182,7 +11178,7 @@
         <v>260</v>
       </c>
       <c r="B59" s="23" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C59" s="56">
         <v>77</v>
@@ -11196,7 +11192,7 @@
         <v>262</v>
       </c>
       <c r="B60" s="23" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C60" s="56">
         <v>79</v>
@@ -11210,7 +11206,7 @@
         <v>264</v>
       </c>
       <c r="B61" s="23" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C61" s="56">
         <v>72</v>
@@ -11224,7 +11220,7 @@
         <v>266</v>
       </c>
       <c r="B62" s="32" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="C62" s="56">
         <v>88</v>
@@ -11238,7 +11234,7 @@
         <v>269</v>
       </c>
       <c r="B63" s="23" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C63" s="56">
         <v>50</v>
@@ -11250,7 +11246,7 @@
         <v>271</v>
       </c>
       <c r="B64" s="52" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C64" s="56">
         <v>79</v>
@@ -11264,7 +11260,7 @@
         <v>274</v>
       </c>
       <c r="B65" s="51" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C65" s="56"/>
       <c r="D65" s="57"/>
@@ -11280,7 +11276,7 @@
         <v>151</v>
       </c>
       <c r="D66" s="65" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="15.95">
@@ -11407,7 +11403,7 @@
       <c r="A76" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="B76" s="10">
+      <c r="B76" s="66">
         <v>1024</v>
       </c>
       <c r="C76" s="56">
@@ -11424,8 +11420,12 @@
       <c r="B77" s="10">
         <v>1536</v>
       </c>
-      <c r="C77" s="56"/>
-      <c r="D77" s="56"/>
+      <c r="C77" s="56">
+        <v>10</v>
+      </c>
+      <c r="D77" s="56">
+        <v>77</v>
+      </c>
     </row>
     <row r="78" spans="1:4" ht="15.95">
       <c r="A78" s="2" t="s">
@@ -11455,7 +11455,9 @@
       <c r="A80" s="2" t="s">
         <v>292</v>
       </c>
-      <c r="B80" s="23"/>
+      <c r="B80" s="32">
+        <v>2000</v>
+      </c>
       <c r="C80" s="56"/>
       <c r="D80" s="56"/>
     </row>
@@ -11463,9 +11465,7 @@
       <c r="A81" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="B81" s="32">
-        <v>2000</v>
-      </c>
+      <c r="B81" s="23"/>
       <c r="C81" s="56"/>
       <c r="D81" s="56"/>
     </row>
@@ -11473,7 +11473,7 @@
       <c r="A82" s="2" t="s">
         <v>294</v>
       </c>
-      <c r="B82" s="23"/>
+      <c r="B82" s="10"/>
       <c r="C82" s="56"/>
       <c r="D82" s="56"/>
     </row>
@@ -11481,30 +11481,36 @@
       <c r="A83" s="2" t="s">
         <v>295</v>
       </c>
-      <c r="B83" s="10"/>
-      <c r="C83" s="56"/>
-      <c r="D83" s="56"/>
+      <c r="B83" s="10">
+        <v>128</v>
+      </c>
+      <c r="C83" s="56">
+        <v>10</v>
+      </c>
+      <c r="D83" s="56">
+        <v>96</v>
+      </c>
     </row>
     <row r="84" spans="1:4" ht="15.95">
       <c r="A84" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="B84" s="10">
-        <v>128</v>
-      </c>
-      <c r="C84" s="56">
+      <c r="B84" s="10" t="s">
+        <v>372</v>
+      </c>
+      <c r="C84" s="10">
         <v>10</v>
       </c>
-      <c r="D84" s="56">
-        <v>96</v>
+      <c r="D84" s="10">
+        <v>84</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.95">
       <c r="A85" s="2" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B85" s="10" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="C85" s="10">
         <v>10</v>
@@ -11515,17 +11521,11 @@
     </row>
     <row r="86" spans="1:4" ht="15.95">
       <c r="A86" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="B86" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="C86" s="10">
-        <v>10</v>
-      </c>
-      <c r="D86" s="10">
-        <v>84</v>
-      </c>
+        <v>300</v>
+      </c>
+      <c r="B86" s="10"/>
+      <c r="C86" s="56"/>
+      <c r="D86" s="56"/>
     </row>
     <row r="87" spans="1:4" ht="15.95">
       <c r="A87" s="2" t="s">
@@ -11547,9 +11547,15 @@
       <c r="A89" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="B89" s="10"/>
-      <c r="C89" s="56"/>
-      <c r="D89" s="56"/>
+      <c r="B89" s="10">
+        <v>96000</v>
+      </c>
+      <c r="C89" s="56">
+        <v>50</v>
+      </c>
+      <c r="D89" s="56">
+        <v>35</v>
+      </c>
     </row>
     <row r="90" spans="1:4" ht="15.95">
       <c r="A90" s="2" t="s">
@@ -11559,7 +11565,7 @@
         <v>96000</v>
       </c>
       <c r="C90" s="56">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="D90" s="56">
         <v>35</v>
@@ -11569,112 +11575,108 @@
       <c r="A91" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="B91" s="10">
+      <c r="B91" s="51">
         <v>96000</v>
       </c>
-      <c r="C91" s="56">
-        <v>55</v>
-      </c>
+      <c r="C91" s="56"/>
       <c r="D91" s="56">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="15.95">
       <c r="A92" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="B92" s="51">
-        <v>96000</v>
-      </c>
-      <c r="C92" s="56"/>
-      <c r="D92" s="106">
+        <v>374</v>
+      </c>
+      <c r="B92" s="26">
+        <v>48000</v>
+      </c>
+      <c r="C92" s="55"/>
+      <c r="D92" s="56">
         <v>41</v>
       </c>
     </row>
-    <row r="93" spans="1:4">
+    <row r="93" spans="1:4" ht="15.95">
       <c r="A93" s="2" t="s">
-        <v>376</v>
-      </c>
-      <c r="B93" s="105">
+        <v>375</v>
+      </c>
+      <c r="B93" s="26">
         <v>48000</v>
       </c>
       <c r="C93" s="55"/>
-      <c r="D93" s="106">
+      <c r="D93" s="56">
         <v>41</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.95">
-      <c r="A94" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="B94" s="26">
-        <v>48000</v>
-      </c>
-      <c r="C94" s="55"/>
+      <c r="A94" s="8" t="s">
+        <v>308</v>
+      </c>
+      <c r="B94" s="35">
+        <v>8000</v>
+      </c>
+      <c r="C94" s="10">
+        <v>99</v>
+      </c>
       <c r="D94" s="56">
         <v>41</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15.95">
-      <c r="A95" s="8" t="s">
+      <c r="A95" s="2" t="s">
+        <v>309</v>
+      </c>
+      <c r="B95" s="68">
+        <v>26000</v>
+      </c>
+      <c r="C95" s="66"/>
+      <c r="D95" s="66" t="s">
         <v>310</v>
       </c>
-      <c r="B95" s="35" t="s">
-        <v>378</v>
-      </c>
-      <c r="C95" s="10">
-        <v>99</v>
-      </c>
-      <c r="D95" s="56">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4">
+    </row>
+    <row r="96" spans="1:4" ht="15.95">
       <c r="A96" s="2" t="s">
         <v>311</v>
       </c>
-      <c r="B96" s="68">
-        <v>26000</v>
-      </c>
-      <c r="C96" s="66"/>
-      <c r="D96" s="66" t="s">
-        <v>312</v>
+      <c r="B96" s="10">
+        <v>1200</v>
+      </c>
+      <c r="C96" s="10">
+        <v>97</v>
+      </c>
+      <c r="D96" s="56">
+        <v>55</v>
       </c>
     </row>
     <row r="97" spans="1:9" ht="15.95">
       <c r="A97" s="2" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B97" s="10">
-        <v>1200</v>
+        <v>500</v>
       </c>
       <c r="C97" s="10">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D97" s="56">
-        <v>55</v>
+        <v>41</v>
       </c>
     </row>
     <row r="98" spans="1:9" ht="15.95">
       <c r="A98" s="2" t="s">
-        <v>314</v>
-      </c>
-      <c r="B98" s="10">
-        <v>500</v>
-      </c>
-      <c r="C98" s="10">
-        <v>99</v>
-      </c>
-      <c r="D98" s="56">
-        <v>41</v>
-      </c>
+        <v>313</v>
+      </c>
+      <c r="B98" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="C98" s="10"/>
+      <c r="D98" s="56"/>
     </row>
     <row r="99" spans="1:9" ht="15.95">
       <c r="A99" s="2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B99" s="10" t="s">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="C99" s="10"/>
       <c r="D99" s="56"/>
@@ -11683,21 +11685,15 @@
       <c r="A100" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="B100" s="10" t="s">
-        <v>380</v>
+      <c r="B100" s="10">
+        <v>10</v>
       </c>
       <c r="C100" s="10"/>
       <c r="D100" s="56"/>
     </row>
-    <row r="101" spans="1:9" ht="15.95">
-      <c r="A101" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="B101" s="10">
-        <v>10</v>
-      </c>
-      <c r="C101" s="10"/>
-      <c r="D101" s="56"/>
+    <row r="101" spans="1:9" ht="15" customHeight="1">
+      <c r="H101" s="11"/>
+      <c r="I101" s="11"/>
     </row>
     <row r="102" spans="1:9" ht="15" customHeight="1">
       <c r="H102" s="11"/>
@@ -11711,12 +11707,8 @@
       <c r="H104" s="11"/>
       <c r="I104" s="11"/>
     </row>
-    <row r="105" spans="1:9" ht="15" customHeight="1">
-      <c r="H105" s="11"/>
-      <c r="I105" s="11"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F101" xr:uid="{63A7BD36-8D88-3742-A4AC-48B0AFB67141}"/>
+  <autoFilter ref="A1:F100" xr:uid="{63A7BD36-8D88-3742-A4AC-48B0AFB67141}"/>
   <mergeCells count="1">
     <mergeCell ref="B1:C1"/>
   </mergeCells>
@@ -11741,7 +11733,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="75">
       <c r="A1" s="75" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="B1" s="103" t="s">
         <v>147</v>
@@ -11751,7 +11743,7 @@
         <v>148</v>
       </c>
       <c r="E1" s="103" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F1" s="104"/>
       <c r="G1" s="76" t="s">
@@ -11760,16 +11752,16 @@
     </row>
     <row r="2" spans="1:7" ht="50.1">
       <c r="A2" s="78" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B2" s="79" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C2" s="80" t="s">
         <v>151</v>
       </c>
       <c r="D2" s="79" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E2" s="79" t="s">
         <v>150</v>
@@ -11783,10 +11775,10 @@
     </row>
     <row r="3" spans="1:7" ht="24.95">
       <c r="A3" s="81" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B3" s="82" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="C3" s="83">
         <v>94</v>
@@ -11795,7 +11787,7 @@
         <v>40</v>
       </c>
       <c r="E3" s="82" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="F3" s="83">
         <v>93</v>
@@ -11806,10 +11798,10 @@
     </row>
     <row r="4" spans="1:7" ht="24.95">
       <c r="A4" s="81" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B4" s="84" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C4" s="85">
         <v>95</v>
@@ -11818,7 +11810,7 @@
         <v>40</v>
       </c>
       <c r="E4" s="84" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F4" s="85">
         <v>94</v>
@@ -11829,7 +11821,7 @@
     </row>
     <row r="5" spans="1:7" ht="24.95">
       <c r="A5" s="81" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B5" s="87" t="s">
         <v>188</v>
@@ -11841,7 +11833,7 @@
         <v>60</v>
       </c>
       <c r="E5" s="87" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="F5" s="88">
         <v>91</v>
@@ -11864,7 +11856,7 @@
         <v>228</v>
       </c>
       <c r="E6" s="84" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F6" s="84">
         <v>98</v>
@@ -11887,7 +11879,7 @@
         <v>228</v>
       </c>
       <c r="E7" s="84" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F7" s="84">
         <v>98</v>
@@ -11910,7 +11902,7 @@
         <v>228</v>
       </c>
       <c r="E8" s="84" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F8" s="84">
         <v>96</v>
@@ -11926,17 +11918,17 @@
       <c r="B9" s="84"/>
       <c r="C9" s="88"/>
       <c r="D9" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E9" s="84"/>
       <c r="F9" s="88"/>
       <c r="G9" s="95" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="75">
-      <c r="A12" s="75" t="s">
-        <v>393</v>
+        <v>389</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="70.5">
+      <c r="A12" s="105" t="s">
+        <v>390</v>
       </c>
       <c r="B12" s="103" t="s">
         <v>147</v>
@@ -11946,7 +11938,7 @@
         <v>148</v>
       </c>
       <c r="E12" s="103" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F12" s="104"/>
       <c r="G12" s="76" t="s">
@@ -11955,16 +11947,16 @@
     </row>
     <row r="13" spans="1:7" ht="50.1">
       <c r="A13" s="78" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B13" s="79" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C13" s="80" t="s">
         <v>151</v>
       </c>
       <c r="D13" s="79" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E13" s="79" t="s">
         <v>150</v>
@@ -11978,10 +11970,10 @@
     </row>
     <row r="14" spans="1:7" ht="24.95">
       <c r="A14" s="81" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B14" s="82" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C14" s="83">
         <v>95</v>
@@ -11990,7 +11982,7 @@
         <v>61</v>
       </c>
       <c r="E14" s="82" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="F14" s="83">
         <v>93</v>
@@ -12001,10 +11993,10 @@
     </row>
     <row r="15" spans="1:7" ht="24.95">
       <c r="A15" s="81" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B15" s="84" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C15" s="85">
         <v>95</v>
@@ -12013,7 +12005,7 @@
         <v>61</v>
       </c>
       <c r="E15" s="84" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F15" s="85">
         <v>94</v>
@@ -12024,7 +12016,7 @@
     </row>
     <row r="16" spans="1:7" ht="24.95">
       <c r="A16" s="81" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B16" s="87" t="s">
         <v>188</v>
@@ -12036,7 +12028,7 @@
         <v>60</v>
       </c>
       <c r="E16" s="87" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="F16" s="88">
         <v>91</v>
@@ -12059,7 +12051,7 @@
         <v>228</v>
       </c>
       <c r="E17" s="84" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F17" s="84">
         <v>98</v>
@@ -12082,7 +12074,7 @@
         <v>228</v>
       </c>
       <c r="E18" s="84" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F18" s="84">
         <v>98</v>
@@ -12105,7 +12097,7 @@
         <v>228</v>
       </c>
       <c r="E19" s="84" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F19" s="84">
         <v>96</v>
@@ -12121,17 +12113,17 @@
       <c r="B20" s="84"/>
       <c r="C20" s="88"/>
       <c r="D20" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E20" s="84"/>
       <c r="F20" s="88"/>
       <c r="G20" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="75">
       <c r="A23" s="96" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="B23" s="103" t="s">
         <v>147</v>
@@ -12141,7 +12133,7 @@
         <v>148</v>
       </c>
       <c r="E23" s="103" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F23" s="104"/>
       <c r="G23" s="76" t="s">
@@ -12150,25 +12142,25 @@
     </row>
     <row r="24" spans="1:9" ht="50.1">
       <c r="A24" s="78" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B24" s="79" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C24" s="80" t="s">
         <v>151</v>
       </c>
       <c r="D24" s="79" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E24" s="79" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F24" s="80" t="s">
         <v>151</v>
       </c>
       <c r="G24" s="79" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="I24" s="77">
         <v>280000</v>
@@ -12176,10 +12168,10 @@
     </row>
     <row r="25" spans="1:9" ht="24.95">
       <c r="A25" s="81" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B25" s="82" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="C25" s="83">
         <v>94</v>
@@ -12188,7 +12180,7 @@
         <v>40</v>
       </c>
       <c r="E25" s="82" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="F25" s="83">
         <v>93</v>
@@ -12203,10 +12195,10 @@
     </row>
     <row r="26" spans="1:9" ht="24.95">
       <c r="A26" s="81" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B26" s="84" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C26" s="85">
         <v>95</v>
@@ -12215,7 +12207,7 @@
         <v>38</v>
       </c>
       <c r="E26" s="84" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F26" s="85">
         <v>94</v>
@@ -12226,10 +12218,10 @@
     </row>
     <row r="27" spans="1:9" ht="24.95">
       <c r="A27" s="81" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B27" s="87" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C27" s="88">
         <v>75</v>
@@ -12238,7 +12230,7 @@
         <v>56</v>
       </c>
       <c r="E27" s="87" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="F27" s="88">
         <v>75</v>
@@ -12247,7 +12239,7 @@
         <v>59</v>
       </c>
       <c r="H27" s="77" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="24.95">
@@ -12264,7 +12256,7 @@
         <v>228</v>
       </c>
       <c r="E28" s="84" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F28" s="84">
         <v>98</v>
@@ -12287,7 +12279,7 @@
         <v>228</v>
       </c>
       <c r="E29" s="84" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F29" s="84">
         <v>98</v>
@@ -12310,7 +12302,7 @@
         <v>228</v>
       </c>
       <c r="E30" s="84" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F30" s="84">
         <v>96</v>
@@ -12330,24 +12322,24 @@
         <v>80</v>
       </c>
       <c r="D31" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E31" s="84" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="F31" s="84">
         <v>77</v>
       </c>
       <c r="G31" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="24.95">
       <c r="A32" s="97" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="B32" s="98" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C32" s="98">
         <v>75</v>
@@ -12356,7 +12348,7 @@
         <v>60</v>
       </c>
       <c r="E32" s="98" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="F32" s="98">
         <v>62</v>
@@ -12365,11 +12357,13 @@
         <v>60</v>
       </c>
       <c r="H32" s="77" t="s">
-        <v>400</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="96"/>
+        <v>397</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="23.25">
+      <c r="A34" s="96" t="s">
+        <v>401</v>
+      </c>
       <c r="B34" s="103" t="s">
         <v>147</v>
       </c>
@@ -12378,7 +12372,7 @@
         <v>148</v>
       </c>
       <c r="E34" s="103" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="F34" s="104"/>
       <c r="G34" s="76" t="s">
@@ -12387,33 +12381,33 @@
     </row>
     <row r="35" spans="1:8" ht="50.1">
       <c r="A35" s="78" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="B35" s="79" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C35" s="80" t="s">
         <v>151</v>
       </c>
       <c r="D35" s="79" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E35" s="79" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="F35" s="80" t="s">
         <v>151</v>
       </c>
       <c r="G35" s="79" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="24.95">
       <c r="A36" s="81" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="B36" s="82" t="s">
-        <v>404</v>
+        <v>402</v>
       </c>
       <c r="C36" s="83">
         <v>93</v>
@@ -12422,7 +12416,7 @@
         <v>40</v>
       </c>
       <c r="E36" s="82" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="F36" s="83">
         <v>95</v>
@@ -12433,10 +12427,10 @@
     </row>
     <row r="37" spans="1:8" ht="24.95">
       <c r="A37" s="81" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="B37" s="84" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="C37" s="85">
         <v>94</v>
@@ -12456,10 +12450,10 @@
     </row>
     <row r="38" spans="1:8" ht="24.95">
       <c r="A38" s="81" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="B38" s="87" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="C38" s="88">
         <v>79</v>
@@ -12468,7 +12462,7 @@
         <v>62</v>
       </c>
       <c r="E38" s="87" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="F38" s="88">
         <v>80</v>
@@ -12477,7 +12471,7 @@
         <v>60</v>
       </c>
       <c r="H38" s="77" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="24.95">
@@ -12494,7 +12488,7 @@
         <v>228</v>
       </c>
       <c r="E39" s="84" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="F39" s="84">
         <v>99</v>
@@ -12517,7 +12511,7 @@
         <v>228</v>
       </c>
       <c r="E40" s="84" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="F40" s="84">
         <v>99</v>
@@ -12540,7 +12534,7 @@
         <v>228</v>
       </c>
       <c r="E41" s="84" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="F41" s="84">
         <v>96</v>
@@ -12560,24 +12554,24 @@
         <v>80</v>
       </c>
       <c r="D42" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="E42" s="84" t="s">
-        <v>409</v>
+        <v>407</v>
       </c>
       <c r="F42" s="84">
         <v>75</v>
       </c>
       <c r="G42" s="95" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="43" spans="1:8" ht="24.95">
       <c r="A43" s="97" t="s">
-        <v>410</v>
+        <v>408</v>
       </c>
       <c r="B43" s="98" t="s">
-        <v>411</v>
+        <v>409</v>
       </c>
       <c r="C43" s="98">
         <v>77</v>
@@ -12586,7 +12580,7 @@
         <v>68</v>
       </c>
       <c r="E43" s="98" t="s">
-        <v>412</v>
+        <v>410</v>
       </c>
       <c r="F43" s="98">
         <v>75</v>
@@ -12595,7 +12589,7 @@
         <v>70</v>
       </c>
       <c r="H43" s="77" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>
@@ -12625,10 +12619,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="60">
       <c r="A1" s="50" t="s">
-        <v>413</v>
+        <v>411</v>
       </c>
       <c r="B1" s="37" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="C1" s="36" t="s">
         <v>148</v>
@@ -12639,34 +12633,34 @@
         <v>149</v>
       </c>
       <c r="B2" s="40" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C2" s="40"/>
     </row>
     <row r="3" spans="1:3" ht="18.95" hidden="1">
       <c r="A3" s="22" t="s">
-        <v>414</v>
+        <v>412</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="42"/>
     </row>
     <row r="4" spans="1:3" ht="15.95" hidden="1">
       <c r="A4" s="2" t="s">
-        <v>415</v>
+        <v>413</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="15.95" hidden="1">
       <c r="A5" s="2" t="s">
-        <v>416</v>
+        <v>414</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="57"/>
     </row>
     <row r="6" spans="1:3" ht="15.95" hidden="1">
       <c r="A6" s="2" t="s">
-        <v>417</v>
+        <v>415</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -12683,10 +12677,10 @@
         <v>160</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>418</v>
+        <v>416</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.95">
@@ -12694,10 +12688,10 @@
         <v>162</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="C9" s="57" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.95" hidden="1">
@@ -12709,7 +12703,7 @@
     </row>
     <row r="11" spans="1:3" ht="15.95" hidden="1">
       <c r="A11" s="2" t="s">
-        <v>422</v>
+        <v>420</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="57"/>
@@ -12730,14 +12724,14 @@
     </row>
     <row r="14" spans="1:3" ht="15.95" hidden="1">
       <c r="A14" s="2" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" ht="15.95" hidden="1">
       <c r="A15" s="2" t="s">
-        <v>424</v>
+        <v>422</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -12751,14 +12745,14 @@
     </row>
     <row r="17" spans="1:3" ht="15.95" hidden="1">
       <c r="A17" s="2" t="s">
-        <v>425</v>
+        <v>423</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" ht="15.95" hidden="1">
       <c r="A18" s="2" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="4"/>
@@ -12772,7 +12766,7 @@
     </row>
     <row r="20" spans="1:3" ht="15.95" hidden="1">
       <c r="A20" s="43" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -12796,10 +12790,10 @@
         <v>187</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>428</v>
+        <v>426</v>
       </c>
       <c r="C23" s="56" t="s">
-        <v>429</v>
+        <v>427</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.95" hidden="1">
@@ -12814,10 +12808,10 @@
         <v>191</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="C25" s="56" t="s">
-        <v>431</v>
+        <v>429</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.95">
@@ -12825,15 +12819,15 @@
         <v>193</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.95" hidden="1">
       <c r="A27" s="2" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="56"/>
@@ -12854,14 +12848,14 @@
     </row>
     <row r="30" spans="1:3" ht="15.95" hidden="1">
       <c r="A30" s="2" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="56"/>
     </row>
     <row r="31" spans="1:3" ht="15.95" hidden="1">
       <c r="A31" s="2" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="B31" s="10"/>
       <c r="C31" s="56"/>
@@ -12927,10 +12921,10 @@
         <v>218</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="C40" s="58" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.95">
@@ -12938,10 +12932,10 @@
         <v>219</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="C41" s="58" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.95" hidden="1">
@@ -12970,10 +12964,10 @@
         <v>223</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15.95" hidden="1">
@@ -13000,32 +12994,32 @@
   <sheetData>
     <row r="1" spans="1:4" ht="81">
       <c r="A1" s="71" t="s">
+        <v>441</v>
+      </c>
+      <c r="B1" s="72" t="s">
+        <v>442</v>
+      </c>
+      <c r="C1" s="73" t="s">
         <v>443</v>
-      </c>
-      <c r="B1" s="72" t="s">
-        <v>444</v>
-      </c>
-      <c r="C1" s="73" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="21.95">
       <c r="A2" s="69" t="s">
+        <v>444</v>
+      </c>
+      <c r="B2" s="70" t="s">
+        <v>445</v>
+      </c>
+      <c r="C2" s="70" t="s">
         <v>446</v>
-      </c>
-      <c r="B2" s="70" t="s">
-        <v>447</v>
-      </c>
-      <c r="C2" s="70" t="s">
-        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95">
       <c r="A3" s="69" t="s">
-        <v>449</v>
+        <v>447</v>
       </c>
       <c r="B3" s="70" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
       <c r="C3" s="70" t="s">
         <v>232</v>
@@ -13033,82 +13027,82 @@
     </row>
     <row r="4" spans="1:4" ht="21.95">
       <c r="A4" s="69" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
       <c r="B4" s="74" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C4" s="74" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="21.95">
       <c r="A5" s="69" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
       <c r="B5" s="74" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="C5" s="74" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="21.95">
       <c r="A6" s="69" t="s">
+        <v>452</v>
+      </c>
+      <c r="B6" s="70" t="s">
+        <v>453</v>
+      </c>
+      <c r="C6" s="70" t="s">
         <v>454</v>
-      </c>
-      <c r="B6" s="70" t="s">
-        <v>455</v>
-      </c>
-      <c r="C6" s="70" t="s">
-        <v>456</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="21.95">
       <c r="A7" s="69" t="s">
+        <v>455</v>
+      </c>
+      <c r="B7" s="70" t="s">
+        <v>456</v>
+      </c>
+      <c r="C7" s="70" t="s">
         <v>457</v>
       </c>
-      <c r="B7" s="70" t="s">
+      <c r="D7" t="s">
         <v>458</v>
-      </c>
-      <c r="C7" s="70" t="s">
-        <v>459</v>
-      </c>
-      <c r="D7" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="21.95">
       <c r="A8" s="69" t="s">
+        <v>459</v>
+      </c>
+      <c r="B8" s="70" t="s">
+        <v>331</v>
+      </c>
+      <c r="C8" s="70" t="s">
+        <v>460</v>
+      </c>
+      <c r="D8" t="s">
         <v>461</v>
-      </c>
-      <c r="B8" s="70" t="s">
-        <v>333</v>
-      </c>
-      <c r="C8" s="70" t="s">
-        <v>462</v>
-      </c>
-      <c r="D8" t="s">
-        <v>463</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="21.95">
       <c r="A9" s="69" t="s">
+        <v>462</v>
+      </c>
+      <c r="B9" s="70" t="s">
+        <v>463</v>
+      </c>
+      <c r="C9" s="70" t="s">
         <v>464</v>
       </c>
-      <c r="B9" s="70" t="s">
+      <c r="D9" t="s">
         <v>465</v>
-      </c>
-      <c r="C9" s="70" t="s">
-        <v>466</v>
-      </c>
-      <c r="D9" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="21.95">
       <c r="A10" s="69" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="B10" s="70">
         <v>26000</v>
@@ -13119,7 +13113,7 @@
     </row>
     <row r="11" spans="1:4" ht="21.95">
       <c r="A11" s="69" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
       <c r="B11" s="70">
         <v>445</v>
@@ -13130,7 +13124,7 @@
     </row>
     <row r="12" spans="1:4" ht="21.95">
       <c r="A12" s="69" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="B12" s="70">
         <v>96000</v>
@@ -13141,7 +13135,7 @@
     </row>
     <row r="13" spans="1:4" ht="21.95">
       <c r="A13" s="69" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="B13" s="70">
         <v>400000</v>
@@ -13152,7 +13146,7 @@
     </row>
     <row r="14" spans="1:4" ht="21.95">
       <c r="A14" s="69" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="B14" s="70">
         <v>200000</v>
@@ -13168,10 +13162,19 @@
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
 <SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="a3ce5a06-b323-45b4-8d97-2f59321c9a5a" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010092711BC64AAEC84E9EF800276F1AD52C" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba397f1440615f1339f1f20b24e67478">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9bf4d24f-a117-48f7-91e1-2035a8c734fd" xmlns:ns3="0b7692b1-2532-40e4-a300-4d7fced4a07a" xmlns:ns4="cb645b5b-9a36-43da-96bf-ab72ec91ddff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="74828cee37efa74eab9b700f6a6651cc" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="9bf4d24f-a117-48f7-91e1-2035a8c734fd"/>
@@ -13419,7 +13422,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="9bf4d24f-a117-48f7-91e1-2035a8c734fd">
@@ -13517,27 +13520,18 @@
 </p:properties>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D75EC423-2542-4A93-99FE-CC28AA840E8C}"/>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4CF876B3-44D4-4080-B40E-3DF67289D40E}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C639165A-13FF-4A9F-A5E9-0E8F0976D502}"/>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E3D764E2-0E35-4957-B738-9033D3F0B0F5}"/>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D75EC423-2542-4A93-99FE-CC28AA840E8C}"/>
 </file>
</xml_diff>

<commit_message>
DS-1: show only tested device for single-device releases
</commit_message>
<xml_diff>
--- a/public/data/SRX4XX_Datasheet.xlsx
+++ b/public/data/SRX4XX_Datasheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hpe-my.sharepoint.com/personal/antony-ruban_alexis_hpe_com/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1038" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7558ED8-9BDD-4EEE-BA08-1951C09F4E01}"/>
+  <xr:revisionPtr revIDLastSave="1059" documentId="8_{1A74DE8B-9E17-7342-8645-B5886219718B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A0D516E-10E4-466C-BD66-8B079F898EC3}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="36000" windowHeight="19740" firstSheet="1" activeTab="2" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="36000" windowHeight="19740" firstSheet="3" activeTab="3" xr2:uid="{982B047A-A65D-41BF-8595-49A5B2074CF1}"/>
   </bookViews>
   <sheets>
     <sheet name="ISSUES-PR's" sheetId="7" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2267" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2294" uniqueCount="473">
   <si>
     <t>number</t>
   </si>
@@ -1296,6 +1296,7 @@
         <sz val="18"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">Release: 25.4X300-202605180407.0-EVO
@@ -1307,6 +1308,7 @@
         <sz val="18"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
+        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
@@ -1394,6 +1396,12 @@
   </si>
   <si>
     <t>345 CPS</t>
+  </si>
+  <si>
+    <t>Release: 25.4X300-202606240112.0-EVO</t>
+  </si>
+  <si>
+    <t>3050 CPS</t>
   </si>
   <si>
     <r>
@@ -1626,7 +1634,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28">
+  <fonts count="27">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1821,18 +1829,9 @@
     </font>
     <font>
       <b/>
-      <u/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="8">
@@ -2099,7 +2098,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="106">
+  <cellXfs count="107">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2383,11 +2382,11 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2395,8 +2394,11 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -8872,10 +8874,10 @@
       <c r="A1" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="105" t="s">
         <v>147</v>
       </c>
-      <c r="C1" s="102"/>
+      <c r="C1" s="106"/>
       <c r="D1" s="36" t="s">
         <v>148</v>
       </c>
@@ -10278,6 +10280,7 @@
     <col min="3" max="3" width="22.140625" style="5" customWidth="1"/>
     <col min="4" max="4" width="46.42578125" customWidth="1"/>
     <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" customWidth="1"/>
     <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10285,10 +10288,10 @@
       <c r="A1" s="50" t="s">
         <v>319</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="105" t="s">
         <v>320</v>
       </c>
-      <c r="C1" s="102"/>
+      <c r="C1" s="106"/>
       <c r="D1" s="36" t="s">
         <v>148</v>
       </c>
@@ -11255,7 +11258,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="32.25" customHeight="1">
+    <row r="65" spans="1:9" ht="32.25" customHeight="1">
       <c r="A65" s="3" t="s">
         <v>274</v>
       </c>
@@ -11265,7 +11268,7 @@
       <c r="C65" s="56"/>
       <c r="D65" s="57"/>
     </row>
-    <row r="66" spans="1:4" ht="18" customHeight="1">
+    <row r="66" spans="1:9" ht="18" customHeight="1">
       <c r="A66" s="28" t="s">
         <v>276</v>
       </c>
@@ -11279,7 +11282,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="67" spans="1:4" ht="15.95">
+    <row r="67" spans="1:9" ht="15.95">
       <c r="A67" s="2" t="s">
         <v>278</v>
       </c>
@@ -11293,7 +11296,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="68" spans="1:4" ht="15.95">
+    <row r="68" spans="1:9" ht="15.95">
       <c r="A68" s="2" t="s">
         <v>279</v>
       </c>
@@ -11306,8 +11309,19 @@
       <c r="D68" s="56">
         <v>76</v>
       </c>
-    </row>
-    <row r="69" spans="1:4" ht="15.95">
+      <c r="G68">
+        <v>123657512</v>
+      </c>
+      <c r="H68">
+        <f>G68/1000</f>
+        <v>123657.512</v>
+      </c>
+      <c r="I68">
+        <f>H68/1000000</f>
+        <v>0.123657512</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="15.95">
       <c r="A69" s="2" t="s">
         <v>280</v>
       </c>
@@ -11315,7 +11329,7 @@
       <c r="C69" s="56"/>
       <c r="D69" s="56"/>
     </row>
-    <row r="70" spans="1:4" ht="15.95">
+    <row r="70" spans="1:9" ht="15.95">
       <c r="A70" s="2" t="s">
         <v>281</v>
       </c>
@@ -11329,7 +11343,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="71" spans="1:4" ht="15.95">
+    <row r="71" spans="1:9" ht="15.95">
       <c r="A71" s="2" t="s">
         <v>282</v>
       </c>
@@ -11343,7 +11357,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="72" spans="1:4" ht="15.95">
+    <row r="72" spans="1:9" ht="15.95">
       <c r="A72" s="2" t="s">
         <v>283</v>
       </c>
@@ -11357,7 +11371,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="73" spans="1:4" ht="15.95">
+    <row r="73" spans="1:9" ht="15.95">
       <c r="A73" s="2" t="s">
         <v>284</v>
       </c>
@@ -11371,7 +11385,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="74" spans="1:4" ht="15.95">
+    <row r="74" spans="1:9" ht="15.95">
       <c r="A74" s="2" t="s">
         <v>286</v>
       </c>
@@ -11385,7 +11399,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="75" spans="1:4" ht="15.95">
+    <row r="75" spans="1:9" ht="15.95">
       <c r="A75" s="2" t="s">
         <v>287</v>
       </c>
@@ -11399,7 +11413,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="15.95">
+    <row r="76" spans="1:9" ht="15.95">
       <c r="A76" s="2" t="s">
         <v>288</v>
       </c>
@@ -11413,7 +11427,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="15.95">
+    <row r="77" spans="1:9" ht="15.95">
       <c r="A77" s="2" t="s">
         <v>289</v>
       </c>
@@ -11427,7 +11441,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="15.95">
+    <row r="78" spans="1:9" ht="15.95">
       <c r="A78" s="2" t="s">
         <v>290</v>
       </c>
@@ -11441,7 +11455,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="15.95">
+    <row r="79" spans="1:9" ht="15.95">
       <c r="A79" s="2" t="s">
         <v>291</v>
       </c>
@@ -11451,7 +11465,7 @@
       <c r="C79" s="56"/>
       <c r="D79" s="56"/>
     </row>
-    <row r="80" spans="1:4" ht="15.95">
+    <row r="80" spans="1:9" ht="15.95">
       <c r="A80" s="2" t="s">
         <v>292</v>
       </c>
@@ -11718,7 +11732,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F1F4FD9-0BA8-D443-A42F-4E5E606C52A0}">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I54"/>
   <sheetFormatPr defaultColWidth="62.42578125" defaultRowHeight="24"/>
   <cols>
     <col min="1" max="1" width="162.42578125" style="77" customWidth="1"/>
@@ -11926,8 +11940,8 @@
         <v>389</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="70.5">
-      <c r="A12" s="105" t="s">
+    <row r="12" spans="1:7" ht="75">
+      <c r="A12" s="75" t="s">
         <v>390</v>
       </c>
       <c r="B12" s="103" t="s">
@@ -12360,7 +12374,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="23.25">
+    <row r="34" spans="1:8" ht="24.95">
       <c r="A34" s="96" t="s">
         <v>401</v>
       </c>
@@ -12592,8 +12606,147 @@
         <v>397</v>
       </c>
     </row>
+    <row r="45" spans="1:8" ht="23.25">
+      <c r="A45" s="101" t="s">
+        <v>411</v>
+      </c>
+      <c r="B45" s="103" t="s">
+        <v>320</v>
+      </c>
+      <c r="C45" s="104"/>
+      <c r="D45" s="76" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="47.25">
+      <c r="A46" s="78" t="s">
+        <v>379</v>
+      </c>
+      <c r="B46" s="79" t="s">
+        <v>336</v>
+      </c>
+      <c r="C46" s="80" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" s="79" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="23.25">
+      <c r="A47" s="81" t="s">
+        <v>381</v>
+      </c>
+      <c r="B47" s="82" t="s">
+        <v>403</v>
+      </c>
+      <c r="C47" s="83">
+        <v>93</v>
+      </c>
+      <c r="D47" s="84">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="23.25">
+      <c r="A48" s="81" t="s">
+        <v>384</v>
+      </c>
+      <c r="B48" s="84" t="s">
+        <v>412</v>
+      </c>
+      <c r="C48" s="85">
+        <v>94</v>
+      </c>
+      <c r="D48" s="86">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="23.25">
+      <c r="A49" s="81" t="s">
+        <v>387</v>
+      </c>
+      <c r="B49" s="87" t="s">
+        <v>406</v>
+      </c>
+      <c r="C49" s="88">
+        <v>80</v>
+      </c>
+      <c r="D49" s="89">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="23.25">
+      <c r="A50" s="90" t="s">
+        <v>226</v>
+      </c>
+      <c r="B50" s="84" t="s">
+        <v>350</v>
+      </c>
+      <c r="C50" s="84">
+        <v>99</v>
+      </c>
+      <c r="D50" s="92" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="23.25">
+      <c r="A51" s="90" t="s">
+        <v>229</v>
+      </c>
+      <c r="B51" s="84" t="s">
+        <v>351</v>
+      </c>
+      <c r="C51" s="84">
+        <v>99</v>
+      </c>
+      <c r="D51" s="92" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="23.25">
+      <c r="A52" s="94" t="s">
+        <v>231</v>
+      </c>
+      <c r="B52" s="84" t="s">
+        <v>352</v>
+      </c>
+      <c r="C52" s="84">
+        <v>96</v>
+      </c>
+      <c r="D52" s="92" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="23.25">
+      <c r="A53" s="81" t="s">
+        <v>260</v>
+      </c>
+      <c r="B53" s="102" t="s">
+        <v>407</v>
+      </c>
+      <c r="C53" s="87">
+        <v>80</v>
+      </c>
+      <c r="D53" s="95" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="23.25">
+      <c r="A54" s="97" t="s">
+        <v>408</v>
+      </c>
+      <c r="B54" s="98" t="s">
+        <v>410</v>
+      </c>
+      <c r="C54" s="98">
+        <v>77</v>
+      </c>
+      <c r="D54" s="98">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="B45:C45"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="E34:F34"/>
     <mergeCell ref="B1:C1"/>
@@ -12619,7 +12772,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="60">
       <c r="A1" s="50" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B1" s="37" t="s">
         <v>320</v>
@@ -12639,28 +12792,28 @@
     </row>
     <row r="3" spans="1:3" ht="18.95" hidden="1">
       <c r="A3" s="22" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B3" s="15"/>
       <c r="C3" s="42"/>
     </row>
     <row r="4" spans="1:3" ht="15.95" hidden="1">
       <c r="A4" s="2" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="4"/>
     </row>
     <row r="5" spans="1:3" ht="15.95" hidden="1">
       <c r="A5" s="2" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="57"/>
     </row>
     <row r="6" spans="1:3" ht="15.95" hidden="1">
       <c r="A6" s="2" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>
@@ -12677,10 +12830,10 @@
         <v>160</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="C8" s="58" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.95">
@@ -12688,10 +12841,10 @@
         <v>162</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="C9" s="57" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.95" hidden="1">
@@ -12703,7 +12856,7 @@
     </row>
     <row r="11" spans="1:3" ht="15.95" hidden="1">
       <c r="A11" s="2" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="57"/>
@@ -12724,14 +12877,14 @@
     </row>
     <row r="14" spans="1:3" ht="15.95" hidden="1">
       <c r="A14" s="2" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B14" s="10"/>
       <c r="C14" s="4"/>
     </row>
     <row r="15" spans="1:3" ht="15.95" hidden="1">
       <c r="A15" s="2" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -12745,14 +12898,14 @@
     </row>
     <row r="17" spans="1:3" ht="15.95" hidden="1">
       <c r="A17" s="2" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4"/>
     </row>
     <row r="18" spans="1:3" ht="15.95" hidden="1">
       <c r="A18" s="2" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="4"/>
@@ -12766,7 +12919,7 @@
     </row>
     <row r="20" spans="1:3" ht="15.95" hidden="1">
       <c r="A20" s="43" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
@@ -12790,10 +12943,10 @@
         <v>187</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="C23" s="56" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="15.95" hidden="1">
@@ -12808,10 +12961,10 @@
         <v>191</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="C25" s="56" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.95">
@@ -12819,15 +12972,15 @@
         <v>193</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="C26" s="56" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="15.95" hidden="1">
       <c r="A27" s="2" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B27" s="10"/>
       <c r="C27" s="56"/>
@@ -12848,14 +13001,14 @@
     </row>
     <row r="30" spans="1:3" ht="15.95" hidden="1">
       <c r="A30" s="2" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B30" s="10"/>
       <c r="C30" s="56"/>
     </row>
     <row r="31" spans="1:3" ht="15.95" hidden="1">
       <c r="A31" s="2" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B31" s="10"/>
       <c r="C31" s="56"/>
@@ -12921,10 +13074,10 @@
         <v>218</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="C40" s="58" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="15.95">
@@ -12932,10 +13085,10 @@
         <v>219</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="C41" s="58" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="15.95" hidden="1">
@@ -12964,10 +13117,10 @@
         <v>223</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="15.95" hidden="1">
@@ -12994,32 +13147,32 @@
   <sheetData>
     <row r="1" spans="1:4" ht="81">
       <c r="A1" s="71" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B1" s="72" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C1" s="73" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="21.95">
       <c r="A2" s="69" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B2" s="70" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="C2" s="70" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="21.95">
       <c r="A3" s="69" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B3" s="70" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="C3" s="70" t="s">
         <v>232</v>
@@ -13027,82 +13180,82 @@
     </row>
     <row r="4" spans="1:4" ht="21.95">
       <c r="A4" s="69" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B4" s="74" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C4" s="74" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="21.95">
       <c r="A5" s="69" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B5" s="74" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C5" s="74" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="21.95">
       <c r="A6" s="69" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B6" s="70" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="C6" s="70" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="21.95">
       <c r="A7" s="69" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B7" s="70" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C7" s="70" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D7" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="21.95">
       <c r="A8" s="69" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B8" s="70" t="s">
         <v>331</v>
       </c>
       <c r="C8" s="70" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="D8" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="21.95">
       <c r="A9" s="69" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B9" s="70" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="D9" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="21.95">
       <c r="A10" s="69" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B10" s="70">
         <v>26000</v>
@@ -13113,7 +13266,7 @@
     </row>
     <row r="11" spans="1:4" ht="21.95">
       <c r="A11" s="69" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B11" s="70">
         <v>445</v>
@@ -13124,7 +13277,7 @@
     </row>
     <row r="12" spans="1:4" ht="21.95">
       <c r="A12" s="69" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B12" s="70">
         <v>96000</v>
@@ -13135,7 +13288,7 @@
     </row>
     <row r="13" spans="1:4" ht="21.95">
       <c r="A13" s="69" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B13" s="70">
         <v>400000</v>
@@ -13146,7 +13299,7 @@
     </row>
     <row r="14" spans="1:4" ht="21.95">
       <c r="A14" s="69" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B14" s="70">
         <v>200000</v>
@@ -13161,20 +13314,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="a3ce5a06-b323-45b4-8d97-2f59321c9a5a" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010092711BC64AAEC84E9EF800276F1AD52C" ma:contentTypeVersion="22" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ba397f1440615f1339f1f20b24e67478">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9bf4d24f-a117-48f7-91e1-2035a8c734fd" xmlns:ns3="0b7692b1-2532-40e4-a300-4d7fced4a07a" xmlns:ns4="cb645b5b-9a36-43da-96bf-ab72ec91ddff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="74828cee37efa74eab9b700f6a6651cc" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="9bf4d24f-a117-48f7-91e1-2035a8c734fd"/>
@@ -13422,6 +13561,20 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="a3ce5a06-b323-45b4-8d97-2f59321c9a5a" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -13521,7 +13674,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D75EC423-2542-4A93-99FE-CC28AA840E8C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C639165A-13FF-4A9F-A5E9-0E8F0976D502}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -13529,7 +13682,7 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C639165A-13FF-4A9F-A5E9-0E8F0976D502}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D75EC423-2542-4A93-99FE-CC28AA840E8C}"/>
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>